<commit_message>
Revised calc. of lwg and growth rates for cattle and pigs
</commit_message>
<xml_diff>
--- a/data/default/PigHerd.xlsx
+++ b/data/default/PigHerd.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\prod_parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="9000" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -1602,6 +1602,29 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1638,29 +1661,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -7456,10 +7456,7 @@
       <c r="H12" t="s">
         <v>30</v>
       </c>
-      <c r="P12" s="13">
-        <f>E3*E5</f>
-        <v>32.571720000000013</v>
-      </c>
+      <c r="P12" s="13"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
@@ -7471,10 +7468,7 @@
       <c r="F13" t="s">
         <v>37</v>
       </c>
-      <c r="P13" s="13">
-        <f>P12*(1-E34/100)*(1-E36/100)</f>
-        <v>26.392688828712011</v>
-      </c>
+      <c r="P13" s="13"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
@@ -9587,19 +9581,19 @@
         <v>69.745999999999995</v>
       </c>
       <c r="Q8" s="132">
-        <f>M8/M$44*100</f>
+        <f t="shared" ref="Q8:Q33" si="3">M8/M$44*100</f>
         <v>39.939446969082496</v>
       </c>
       <c r="R8" s="98">
-        <f>N8/N$44*100</f>
+        <f t="shared" ref="R8:R33" si="4">N8/N$44*100</f>
         <v>37.344664381805039</v>
       </c>
       <c r="S8" s="134">
-        <f>O8/O$44*100</f>
+        <f t="shared" ref="S8:S33" si="5">O8/O$44*100</f>
         <v>31.302145183860713</v>
       </c>
       <c r="T8" s="102">
-        <f>O8/O$44*100</f>
+        <f t="shared" ref="T8:T33" si="6">O8/O$44*100</f>
         <v>31.302145183860713</v>
       </c>
       <c r="U8" s="98"/>
@@ -9651,19 +9645,19 @@
         <v>53.577999999999996</v>
       </c>
       <c r="Q9" s="132">
-        <f>M9/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>33.588951440574981</v>
       </c>
       <c r="R9" s="98">
-        <f>N9/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>33.835769741903896</v>
       </c>
       <c r="S9" s="98">
-        <f>O9/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>24.045914241116183</v>
       </c>
       <c r="T9" s="102">
-        <f>O9/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>24.045914241116183</v>
       </c>
       <c r="U9" s="98"/>
@@ -9715,19 +9709,19 @@
         <v>9.0299999999999994</v>
       </c>
       <c r="Q10" s="132">
-        <f>M10/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>4.876686724200181</v>
       </c>
       <c r="R10" s="98">
-        <f>N10/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>7.2684246112238</v>
       </c>
       <c r="S10" s="98">
-        <f>O10/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>4.0526821754690197</v>
       </c>
       <c r="T10" s="102">
-        <f>O10/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>4.0526821754690197</v>
       </c>
       <c r="U10" s="98"/>
@@ -9767,31 +9761,31 @@
         <v>162</v>
       </c>
       <c r="M11" s="97">
-        <f>D11*($J11/100)</f>
+        <f t="shared" ref="M11:M21" si="7">D11*($J11/100)</f>
         <v>4.9879999999999995</v>
       </c>
       <c r="N11" s="99">
-        <f>F11*($J11/100)</f>
+        <f t="shared" ref="N11:N21" si="8">F11*($J11/100)</f>
         <v>0</v>
       </c>
       <c r="O11" s="130">
-        <f>H11*($J11/100)</f>
+        <f t="shared" ref="O11:O21" si="9">H11*($J11/100)</f>
         <v>8.4280000000000008</v>
       </c>
       <c r="Q11" s="132">
-        <f>M11/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.44754403481583932</v>
       </c>
       <c r="R11" s="98">
-        <f>N11/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S11" s="98">
-        <f>O11/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>3.7825033637710859</v>
       </c>
       <c r="T11" s="102">
-        <f>O11/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>3.7825033637710859</v>
       </c>
       <c r="U11" s="98"/>
@@ -9831,31 +9825,31 @@
         <v>165</v>
       </c>
       <c r="M12" s="97">
-        <f>D12*($J12/100)</f>
+        <f t="shared" si="7"/>
         <v>2.4939999999999998</v>
       </c>
       <c r="N12" s="99">
-        <f>F12*($J12/100)</f>
+        <f t="shared" si="8"/>
         <v>0.60199999999999998</v>
       </c>
       <c r="O12" s="130">
-        <f>H12*($J12/100)</f>
+        <f t="shared" si="9"/>
         <v>0.17200000000000001</v>
       </c>
       <c r="Q12" s="132">
-        <f>M12/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.22377201740791966</v>
       </c>
       <c r="R12" s="98">
-        <f>N12/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>1.7544473199505721</v>
       </c>
       <c r="S12" s="98">
-        <f>O12/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>7.7193946199409905E-2</v>
       </c>
       <c r="T12" s="102">
-        <f>O12/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>7.7193946199409905E-2</v>
       </c>
       <c r="U12" s="98"/>
@@ -9895,31 +9889,31 @@
         <v>218</v>
       </c>
       <c r="M13" s="97">
-        <f>D13*($J13/100)</f>
+        <f t="shared" si="7"/>
         <v>8.7550000000000008</v>
       </c>
       <c r="N13" s="99">
-        <f>F13*($J13/100)</f>
+        <f t="shared" si="8"/>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="O13" s="130">
-        <f>H13*($J13/100)</f>
+        <f t="shared" si="9"/>
         <v>1.02</v>
       </c>
       <c r="Q13" s="132">
-        <f>M13/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.78553488869540378</v>
       </c>
       <c r="R13" s="98">
-        <f>N13/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0.24772096710265556</v>
       </c>
       <c r="S13" s="98">
-        <f>O13/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0.45777805304301217</v>
       </c>
       <c r="T13" s="102">
-        <f>O13/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0.45777805304301217</v>
       </c>
       <c r="U13" s="98"/>
@@ -9959,31 +9953,31 @@
         <v>219</v>
       </c>
       <c r="M14" s="97">
-        <f>D14*($J14/100)</f>
+        <f t="shared" si="7"/>
         <v>1.105</v>
       </c>
       <c r="N14" s="99">
-        <f>F14*($J14/100)</f>
+        <f t="shared" si="8"/>
         <v>0.255</v>
       </c>
       <c r="O14" s="130">
-        <f>H14*($J14/100)</f>
+        <f t="shared" si="9"/>
         <v>17.254999999999999</v>
       </c>
       <c r="Q14" s="132">
-        <f>M14/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>9.9145180126604351E-2</v>
       </c>
       <c r="R14" s="98">
-        <f>N14/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0.74316290130796658</v>
       </c>
       <c r="S14" s="98">
-        <f>O14/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>7.74407873064429</v>
       </c>
       <c r="T14" s="102">
-        <f>O14/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>7.74407873064429</v>
       </c>
       <c r="U14" s="98"/>
@@ -10023,31 +10017,31 @@
         <v>163</v>
       </c>
       <c r="M15" s="97">
-        <f>D15*($J15/100)</f>
+        <f t="shared" si="7"/>
         <v>3.9129999999999998</v>
       </c>
       <c r="N15" s="99">
-        <f>F15*($J15/100)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O15" s="130">
-        <f>H15*($J15/100)</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q15" s="132">
-        <f>M15/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.35109057903656365</v>
       </c>
       <c r="R15" s="98">
-        <f>N15/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S15" s="98">
-        <f>O15/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T15" s="102">
-        <f>O15/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U15" s="98"/>
@@ -10087,31 +10081,31 @@
         <v>164</v>
       </c>
       <c r="M16" s="97">
-        <f>D16*($J16/100)</f>
+        <f t="shared" si="7"/>
         <v>1.4560000000000002</v>
       </c>
       <c r="N16" s="99">
-        <f>F16*($J16/100)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O16" s="130">
-        <f>H16*($J16/100)</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q16" s="132">
-        <f>M16/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.13063835499034929</v>
       </c>
       <c r="R16" s="98">
-        <f>N16/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S16" s="98">
-        <f>O16/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T16" s="102">
-        <f>O16/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U16" s="98"/>
@@ -10151,31 +10145,31 @@
         <v>220</v>
       </c>
       <c r="M17" s="97">
-        <f>D17*($J17/100)</f>
+        <f t="shared" si="7"/>
         <v>77.967999999999989</v>
       </c>
       <c r="N17" s="99">
-        <f>F17*($J17/100)</f>
+        <f t="shared" si="8"/>
         <v>2.464</v>
       </c>
       <c r="O17" s="130">
-        <f>H17*($J17/100)</f>
+        <f t="shared" si="9"/>
         <v>6.3360000000000003</v>
       </c>
       <c r="Q17" s="132">
-        <f>M17/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>6.9956121304172738</v>
       </c>
       <c r="R17" s="98">
-        <f>N17/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>7.1809936816581557</v>
       </c>
       <c r="S17" s="98">
-        <f>O17/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>2.8436095530201233</v>
       </c>
       <c r="T17" s="102">
-        <f>O17/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>2.8436095530201233</v>
       </c>
       <c r="U17" s="98"/>
@@ -10215,31 +10209,31 @@
         <v>222</v>
       </c>
       <c r="M18" s="97">
-        <f>D18*($J18/100)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="N18" s="99">
-        <f>F18*($J18/100)</f>
+        <f t="shared" si="8"/>
         <v>0.78300000000000003</v>
       </c>
       <c r="O18" s="130">
-        <f>H18*($J18/100)</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q18" s="132">
-        <f>M18/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R18" s="98">
-        <f>N18/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>2.2819472616632859</v>
       </c>
       <c r="S18" s="98">
-        <f>O18/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T18" s="102">
-        <f>O18/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U18" s="98"/>
@@ -10279,31 +10273,31 @@
         <v>221</v>
       </c>
       <c r="M19" s="97">
-        <f>D19*($J19/100)</f>
+        <f t="shared" si="7"/>
         <v>36.630000000000003</v>
       </c>
       <c r="N19" s="99">
-        <f>F19*($J19/100)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O19" s="130">
-        <f>H19*($J19/100)</f>
+        <f t="shared" si="9"/>
         <v>7.8299999999999992</v>
       </c>
       <c r="Q19" s="132">
-        <f>M19/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>3.2865954280882512</v>
       </c>
       <c r="R19" s="98">
-        <f>N19/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S19" s="98">
-        <f>O19/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>3.5141197601242991</v>
       </c>
       <c r="T19" s="102">
-        <f>O19/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>3.5141197601242991</v>
       </c>
       <c r="U19" s="98"/>
@@ -10343,31 +10337,31 @@
         <v>217</v>
       </c>
       <c r="M20" s="97">
-        <f>D20*($J20/100)</f>
+        <f t="shared" si="7"/>
         <v>5.0049999999999999</v>
       </c>
       <c r="N20" s="99">
-        <f>F20*($J20/100)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O20" s="130">
-        <f>H20*($J20/100)</f>
+        <f t="shared" si="9"/>
         <v>0.36400000000000005</v>
       </c>
       <c r="Q20" s="132">
-        <f>M20/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.44906934527932563</v>
       </c>
       <c r="R20" s="98">
-        <f>N20/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S20" s="98">
-        <f>O20/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0.16336393265456514</v>
       </c>
       <c r="T20" s="102">
-        <f>O20/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0.16336393265456514</v>
       </c>
       <c r="U20" s="98"/>
@@ -10407,31 +10401,31 @@
         <v>213</v>
       </c>
       <c r="M21" s="97">
-        <f>D21*($J21/100)</f>
+        <f t="shared" si="7"/>
         <v>1.4560000000000002</v>
       </c>
       <c r="N21" s="99">
-        <f>F21*($J21/100)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O21" s="130">
-        <f>H21*($J21/100)</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q21" s="132">
-        <f>M21/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.13063835499034929</v>
       </c>
       <c r="R21" s="98">
-        <f>N21/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S21" s="98">
-        <f>O21/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T21" s="102">
-        <f>O21/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U21" s="98"/>
@@ -10483,19 +10477,19 @@
         <v>18.443999999999999</v>
       </c>
       <c r="Q22" s="132">
-        <f>M22/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>3.1145942422939523</v>
       </c>
       <c r="R22" s="98">
-        <f>N22/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S22" s="98">
-        <f>O22/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>8.277704323848349</v>
       </c>
       <c r="T22" s="102">
-        <f>O22/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>8.277704323848349</v>
       </c>
       <c r="U22" s="98"/>
@@ -10550,19 +10544,19 @@
         <v>1.9360000000000002</v>
       </c>
       <c r="Q23" s="132">
-        <f>M23/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>2.3450302513926982</v>
       </c>
       <c r="R23" s="98">
-        <f>N23/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>1.2823203002960992</v>
       </c>
       <c r="S23" s="98">
-        <f>O23/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0.86888069675614876</v>
       </c>
       <c r="T23" s="102">
-        <f>O23/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0.86888069675614876</v>
       </c>
       <c r="U23" s="98"/>
@@ -10614,19 +10608,19 @@
         <v>0.36000000000000004</v>
       </c>
       <c r="Q24" s="132">
-        <f>M24/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.13727794171375987</v>
       </c>
       <c r="R24" s="98">
-        <f>N24/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S24" s="98">
-        <f>O24/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0.16156872460341609</v>
       </c>
       <c r="T24" s="102">
-        <f>O24/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0.16156872460341609</v>
       </c>
       <c r="U24" s="98"/>
@@ -10678,19 +10672,19 @@
         <v>10.4574</v>
       </c>
       <c r="Q25" s="132">
-        <f>M25/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.59612721878837949</v>
       </c>
       <c r="R25" s="98">
-        <f>N25/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S25" s="98">
-        <f>O25/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>4.6933021685215648</v>
       </c>
       <c r="T25" s="102">
-        <f>O25/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>4.6933021685215648</v>
       </c>
       <c r="U25" s="98"/>
@@ -10742,19 +10736,19 @@
         <v>0.22799999999999998</v>
       </c>
       <c r="Q26" s="132">
-        <f>M26/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.35458982068809092</v>
       </c>
       <c r="R26" s="98">
-        <f>N26/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S26" s="98">
-        <f>O26/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0.10232685891549684</v>
       </c>
       <c r="T26" s="102">
-        <f>O26/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0.10232685891549684</v>
       </c>
       <c r="U26" s="98"/>
@@ -10806,19 +10800,19 @@
         <v>0</v>
       </c>
       <c r="Q27" s="132">
-        <f>M27/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.69473405404551813</v>
       </c>
       <c r="R27" s="98">
-        <f>N27/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S27" s="98">
-        <f>O27/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T27" s="102">
-        <f>O27/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U27" s="98"/>
@@ -10870,19 +10864,19 @@
         <v>9.7110000000000003</v>
       </c>
       <c r="Q28" s="132">
-        <f>M28/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>1.0649538207770974</v>
       </c>
       <c r="R28" s="98">
-        <f>N28/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>1.7626075400433656</v>
       </c>
       <c r="S28" s="98">
-        <f>O28/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>4.3583163461771495</v>
       </c>
       <c r="T28" s="102">
-        <f>O28/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>4.3583163461771495</v>
       </c>
       <c r="U28" s="98"/>
@@ -10934,19 +10928,19 @@
         <v>0</v>
       </c>
       <c r="Q29" s="132">
-        <f>M29/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R29" s="98">
-        <f>N29/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0.2826933389289128</v>
       </c>
       <c r="S29" s="98">
-        <f>O29/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T29" s="102">
-        <f>O29/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U29" s="98"/>
@@ -10998,19 +10992,19 @@
         <v>0</v>
       </c>
       <c r="Q30" s="132">
-        <f>M30/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R30" s="98">
-        <f>N30/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>1.3406075866731948</v>
       </c>
       <c r="S30" s="98">
-        <f>O30/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T30" s="102">
-        <f>O30/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U30" s="98"/>
@@ -11062,19 +11056,19 @@
         <v>0</v>
       </c>
       <c r="Q31" s="132">
-        <f>M31/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.18160166929977128</v>
       </c>
       <c r="R31" s="98">
-        <f>N31/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>3.2174582080156675</v>
       </c>
       <c r="S31" s="98">
-        <f>O31/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T31" s="102">
-        <f>O31/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U31" s="98"/>
@@ -11126,19 +11120,19 @@
         <v>0</v>
       </c>
       <c r="Q32" s="132">
-        <f>M32/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0.20636553329519458</v>
       </c>
       <c r="R32" s="98">
-        <f>N32/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>1.4571821594273857</v>
       </c>
       <c r="S32" s="98">
-        <f>O32/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T32" s="102">
-        <f>O32/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U32" s="98"/>
@@ -11147,27 +11141,27 @@
       <c r="B33" s="87" t="s">
         <v>243</v>
       </c>
-      <c r="C33" s="156" t="s">
+      <c r="C33" s="141" t="s">
         <v>172</v>
       </c>
-      <c r="D33" s="157">
+      <c r="D33" s="142">
         <v>62.6</v>
       </c>
-      <c r="E33" s="158">
+      <c r="E33" s="143">
         <f t="shared" si="0"/>
         <v>3.8430842900116641E-2</v>
       </c>
-      <c r="F33" s="157">
+      <c r="F33" s="142">
         <v>1.8</v>
       </c>
-      <c r="G33" s="158">
+      <c r="G33" s="143">
         <f t="shared" si="1"/>
         <v>3.272727272727273E-2</v>
       </c>
-      <c r="H33" s="157">
+      <c r="H33" s="142">
         <v>11</v>
       </c>
-      <c r="I33" s="159">
+      <c r="I33" s="144">
         <f t="shared" si="2"/>
         <v>2.1480179652411637E-2</v>
       </c>
@@ -11188,19 +11182,19 @@
         <v>7.9200000000000008</v>
       </c>
       <c r="Q33" s="132">
-        <f>M33/M$44*100</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R33" s="98">
-        <f>N33/N$44*100</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="S33" s="98">
-        <f>O33/O$44*100</f>
+        <f t="shared" si="5"/>
         <v>3.554511941275154</v>
       </c>
       <c r="T33" s="102">
-        <f>O33/O$44*100</f>
+        <f t="shared" si="6"/>
         <v>3.554511941275154</v>
       </c>
       <c r="U33" s="98"/>
@@ -11209,27 +11203,27 @@
       <c r="B34" s="87" t="s">
         <v>243</v>
       </c>
-      <c r="C34" s="156" t="s">
+      <c r="C34" s="141" t="s">
         <v>186</v>
       </c>
-      <c r="D34" s="157">
+      <c r="D34" s="142">
         <v>5.8</v>
       </c>
-      <c r="E34" s="158">
+      <c r="E34" s="143">
         <f t="shared" si="0"/>
         <v>3.5606851249309346E-3</v>
       </c>
-      <c r="F34" s="157">
+      <c r="F34" s="142">
         <v>0.2</v>
       </c>
-      <c r="G34" s="158">
+      <c r="G34" s="143">
         <f t="shared" si="1"/>
         <v>3.6363636363636364E-3</v>
       </c>
-      <c r="H34" s="157">
+      <c r="H34" s="142">
         <v>1.4</v>
       </c>
-      <c r="I34" s="159">
+      <c r="I34" s="144">
         <f t="shared" si="2"/>
         <v>2.7338410466705718E-3</v>
       </c>
@@ -11247,27 +11241,27 @@
       <c r="B35" s="87" t="s">
         <v>243</v>
       </c>
-      <c r="C35" s="156" t="s">
+      <c r="C35" s="141" t="s">
         <v>201</v>
       </c>
-      <c r="D35" s="157">
+      <c r="D35" s="142">
         <v>43.3</v>
       </c>
-      <c r="E35" s="158">
+      <c r="E35" s="143">
         <f t="shared" si="0"/>
         <v>2.6582356191294735E-2</v>
       </c>
-      <c r="F35" s="157">
+      <c r="F35" s="142">
         <v>4.5</v>
       </c>
-      <c r="G35" s="158">
+      <c r="G35" s="143">
         <f t="shared" si="1"/>
         <v>8.1818181818181818E-2</v>
       </c>
-      <c r="H35" s="157">
-        <v>0</v>
-      </c>
-      <c r="I35" s="159">
+      <c r="H35" s="142">
+        <v>0</v>
+      </c>
+      <c r="I35" s="144">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -11446,27 +11440,27 @@
       <c r="B40" s="87" t="s">
         <v>243</v>
       </c>
-      <c r="C40" s="160" t="s">
+      <c r="C40" s="145" t="s">
         <v>205</v>
       </c>
-      <c r="D40" s="157">
-        <v>0</v>
-      </c>
-      <c r="E40" s="158">
+      <c r="D40" s="142">
+        <v>0</v>
+      </c>
+      <c r="E40" s="143">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F40" s="157">
-        <v>0</v>
-      </c>
-      <c r="G40" s="158">
+      <c r="F40" s="142">
+        <v>0</v>
+      </c>
+      <c r="G40" s="143">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H40" s="157">
+      <c r="H40" s="142">
         <v>15.7</v>
       </c>
-      <c r="I40" s="159">
+      <c r="I40" s="144">
         <f t="shared" si="2"/>
         <v>3.0658074594805698E-2</v>
       </c>
@@ -11526,27 +11520,27 @@
       <c r="B42" s="87" t="s">
         <v>243</v>
       </c>
-      <c r="C42" s="161" t="s">
+      <c r="C42" s="146" t="s">
         <v>207</v>
       </c>
-      <c r="D42" s="162">
-        <v>0</v>
-      </c>
-      <c r="E42" s="163">
+      <c r="D42" s="147">
+        <v>0</v>
+      </c>
+      <c r="E42" s="148">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F42" s="162">
-        <v>0</v>
-      </c>
-      <c r="G42" s="163">
+      <c r="F42" s="147">
+        <v>0</v>
+      </c>
+      <c r="G42" s="148">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H42" s="162">
+      <c r="H42" s="147">
         <v>4.7</v>
       </c>
-      <c r="I42" s="164">
+      <c r="I42" s="149">
         <f t="shared" si="2"/>
         <v>9.1778949423940628E-3</v>
       </c>
@@ -11623,15 +11617,15 @@
         <v>100</v>
       </c>
       <c r="R44" s="133">
-        <f t="shared" ref="R44:T44" si="3">SUM(R8:R43)</f>
+        <f t="shared" ref="R44:T44" si="10">SUM(R8:R43)</f>
         <v>100</v>
       </c>
       <c r="S44" s="133">
-        <f t="shared" si="3"/>
+        <f t="shared" si="10"/>
         <v>100</v>
       </c>
       <c r="T44" s="124">
-        <f t="shared" si="3"/>
+        <f t="shared" si="10"/>
         <v>100</v>
       </c>
       <c r="U44" s="129"/>
@@ -11694,7 +11688,7 @@
       <c r="O50" s="87"/>
     </row>
     <row r="51" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C51" s="150" t="s">
+      <c r="C51" s="138" t="s">
         <v>245</v>
       </c>
       <c r="D51" s="118"/>
@@ -11702,20 +11696,20 @@
       <c r="F51" s="118"/>
       <c r="G51" s="118"/>
       <c r="H51" s="118"/>
-      <c r="I51" s="151"/>
+      <c r="I51" s="139"/>
       <c r="J51" s="78"/>
     </row>
     <row r="52" spans="3:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="152" t="s">
+      <c r="C52" s="150" t="s">
         <v>244</v>
       </c>
-      <c r="D52" s="153"/>
-      <c r="E52" s="153"/>
-      <c r="F52" s="153"/>
-      <c r="G52" s="153"/>
-      <c r="H52" s="153"/>
-      <c r="I52" s="154"/>
-      <c r="J52" s="155"/>
+      <c r="D52" s="151"/>
+      <c r="E52" s="151"/>
+      <c r="F52" s="151"/>
+      <c r="G52" s="151"/>
+      <c r="H52" s="151"/>
+      <c r="I52" s="152"/>
+      <c r="J52" s="140"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -13974,19 +13968,19 @@
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="40"/>
-      <c r="C23" s="144" t="s">
+      <c r="C23" s="159" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="146" t="s">
+      <c r="D23" s="161" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="139" t="s">
+      <c r="E23" s="154" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="141" t="s">
+      <c r="F23" s="156" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="143"/>
+      <c r="G23" s="158"/>
       <c r="H23" s="31"/>
       <c r="O23">
         <v>11</v>
@@ -14008,11 +14002,11 @@
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" s="41"/>
-      <c r="C24" s="145"/>
-      <c r="D24" s="147"/>
-      <c r="E24" s="140"/>
-      <c r="F24" s="142"/>
-      <c r="G24" s="143"/>
+      <c r="C24" s="160"/>
+      <c r="D24" s="162"/>
+      <c r="E24" s="155"/>
+      <c r="F24" s="157"/>
+      <c r="G24" s="158"/>
       <c r="H24" s="18"/>
       <c r="O24">
         <v>13</v>
@@ -14033,13 +14027,13 @@
       </c>
     </row>
     <row r="25" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="149" t="s">
+      <c r="B25" s="164" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="149"/>
-      <c r="D25" s="149"/>
-      <c r="E25" s="149"/>
-      <c r="F25" s="149"/>
+      <c r="C25" s="164"/>
+      <c r="D25" s="164"/>
+      <c r="E25" s="164"/>
+      <c r="F25" s="164"/>
       <c r="G25" s="42"/>
       <c r="H25" s="18"/>
       <c r="O25">
@@ -14061,13 +14055,13 @@
       </c>
     </row>
     <row r="26" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="138" t="s">
+      <c r="B26" s="153" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="138"/>
-      <c r="D26" s="138"/>
-      <c r="E26" s="138"/>
-      <c r="F26" s="138"/>
+      <c r="C26" s="153"/>
+      <c r="D26" s="153"/>
+      <c r="E26" s="153"/>
+      <c r="F26" s="153"/>
       <c r="G26" s="42"/>
       <c r="H26" s="18"/>
       <c r="O26">
@@ -14259,25 +14253,25 @@
       <c r="R33" s="3"/>
     </row>
     <row r="34" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="148" t="s">
+      <c r="B34" s="163" t="s">
         <v>8</v>
       </c>
-      <c r="C34" s="148"/>
-      <c r="D34" s="148"/>
-      <c r="E34" s="148"/>
-      <c r="F34" s="148"/>
+      <c r="C34" s="163"/>
+      <c r="D34" s="163"/>
+      <c r="E34" s="163"/>
+      <c r="F34" s="163"/>
       <c r="G34" s="42"/>
       <c r="H34" s="18"/>
       <c r="R34" s="13"/>
     </row>
     <row r="35" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="138" t="s">
+      <c r="B35" s="153" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="138"/>
-      <c r="D35" s="138"/>
-      <c r="E35" s="138"/>
-      <c r="F35" s="138"/>
+      <c r="C35" s="153"/>
+      <c r="D35" s="153"/>
+      <c r="E35" s="153"/>
+      <c r="F35" s="153"/>
       <c r="G35" s="42"/>
       <c r="H35" s="18"/>
     </row>

</xml_diff>

<commit_message>
Implemented calculation of bedding material use and its NPK addition to manure
</commit_message>
<xml_diff>
--- a/data/default/PigHerd.xlsx
+++ b/data/default/PigHerd.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Slaktstat" sheetId="3" r:id="rId4"/>
     <sheet name="Sheet2" sheetId="7" r:id="rId5"/>
     <sheet name="Energi rek" sheetId="5" r:id="rId6"/>
+    <sheet name="references" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="247">
   <si>
     <t>parameter</t>
   </si>
@@ -509,9 +510,6 @@
   </si>
   <si>
     <t>Fallback</t>
-  </si>
-  <si>
-    <t>Landquist et al. 2020. Uppdaterad och utökad livscykelanalys av svensk grisproduktion</t>
   </si>
   <si>
     <t>barley</t>
@@ -816,6 +814,12 @@
   </si>
   <si>
     <t>E-mail from Birgit Landquist (RISE) 2023-10-16</t>
+  </si>
+  <si>
+    <t>Landquist et al. 2020. Uppdaterad och utökad livscykelanalys av svensk grisproduktion. RISE</t>
+  </si>
+  <si>
+    <t>Landquist et al. 2020</t>
   </si>
 </sst>
 </file>
@@ -1710,6 +1714,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -1839,6 +1844,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -1872,6 +1878,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -1925,6 +1932,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2054,6 +2062,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2087,6 +2096,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2140,6 +2150,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2362,6 +2373,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2395,6 +2407,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -2408,6 +2421,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2452,6 +2466,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2674,6 +2689,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2707,6 +2723,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -2720,6 +2737,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2764,6 +2782,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2893,6 +2912,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2926,6 +2946,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2964,6 +2985,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3360,6 +3382,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3726,6 +3749,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4097,6 +4121,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -8038,7 +8063,7 @@
         <v>154</v>
       </c>
       <c r="H50" t="s">
-        <v>159</v>
+        <v>246</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -8096,10 +8121,10 @@
       <c r="E54" s="8"/>
       <c r="F54" s="8"/>
       <c r="G54" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>159</v>
+        <v>246</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -8167,7 +8192,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="93" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B60" s="93"/>
       <c r="C60" s="93"/>
@@ -8194,7 +8219,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C62" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D62" t="s">
         <v>71</v>
@@ -8209,7 +8234,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C63" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D63" t="s">
         <v>71</v>
@@ -8224,7 +8249,7 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C64" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D64" t="s">
         <v>71</v>
@@ -8239,7 +8264,7 @@
     </row>
     <row r="65" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D65" t="s">
         <v>71</v>
@@ -8254,7 +8279,7 @@
     </row>
     <row r="66" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D66" t="s">
         <v>71</v>
@@ -8269,7 +8294,7 @@
     </row>
     <row r="67" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C67" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D67" t="s">
         <v>71</v>
@@ -8284,7 +8309,7 @@
     </row>
     <row r="68" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D68" t="s">
         <v>71</v>
@@ -8299,7 +8324,7 @@
     </row>
     <row r="69" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -8314,7 +8339,7 @@
     </row>
     <row r="70" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D70" t="s">
         <v>71</v>
@@ -8329,7 +8354,7 @@
     </row>
     <row r="71" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D71" t="s">
         <v>71</v>
@@ -8344,7 +8369,7 @@
     </row>
     <row r="72" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C72" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D72" t="s">
         <v>71</v>
@@ -8359,7 +8384,7 @@
     </row>
     <row r="73" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C73" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D73" t="s">
         <v>71</v>
@@ -8374,7 +8399,7 @@
     </row>
     <row r="74" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C74" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D74" t="s">
         <v>71</v>
@@ -8389,7 +8414,7 @@
     </row>
     <row r="75" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D75" t="s">
         <v>71</v>
@@ -8404,7 +8429,7 @@
     </row>
     <row r="76" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D76" t="s">
         <v>71</v>
@@ -8419,7 +8444,7 @@
     </row>
     <row r="77" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D77" t="s">
         <v>71</v>
@@ -8434,7 +8459,7 @@
     </row>
     <row r="78" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C78" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D78" t="s">
         <v>71</v>
@@ -8449,7 +8474,7 @@
     </row>
     <row r="79" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D79" t="s">
         <v>71</v>
@@ -8464,7 +8489,7 @@
     </row>
     <row r="80" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D80" t="s">
         <v>71</v>
@@ -8479,7 +8504,7 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D81" t="s">
         <v>71</v>
@@ -8494,7 +8519,7 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D82" t="s">
         <v>71</v>
@@ -8509,7 +8534,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="93" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B83" s="93"/>
       <c r="C83" s="93"/>
@@ -8542,7 +8567,7 @@
         <v>15</v>
       </c>
       <c r="C85" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D85" t="s">
         <v>71</v>
@@ -8560,7 +8585,7 @@
         <v>15</v>
       </c>
       <c r="C86" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D86" t="s">
         <v>71</v>
@@ -8578,7 +8603,7 @@
         <v>15</v>
       </c>
       <c r="C87" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D87" t="s">
         <v>71</v>
@@ -8596,7 +8621,7 @@
         <v>15</v>
       </c>
       <c r="C88" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D88" t="s">
         <v>71</v>
@@ -8614,7 +8639,7 @@
         <v>15</v>
       </c>
       <c r="C89" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D89" t="s">
         <v>71</v>
@@ -8632,7 +8657,7 @@
         <v>15</v>
       </c>
       <c r="C90" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D90" t="s">
         <v>71</v>
@@ -8650,7 +8675,7 @@
         <v>15</v>
       </c>
       <c r="C91" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D91" t="s">
         <v>71</v>
@@ -8668,7 +8693,7 @@
         <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D92" t="s">
         <v>71</v>
@@ -8686,7 +8711,7 @@
         <v>15</v>
       </c>
       <c r="C93" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D93" t="s">
         <v>71</v>
@@ -8704,7 +8729,7 @@
         <v>15</v>
       </c>
       <c r="C94" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D94" t="s">
         <v>71</v>
@@ -8722,7 +8747,7 @@
         <v>15</v>
       </c>
       <c r="C95" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D95" t="s">
         <v>71</v>
@@ -8740,7 +8765,7 @@
         <v>15</v>
       </c>
       <c r="C96" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D96" t="s">
         <v>71</v>
@@ -8758,7 +8783,7 @@
         <v>15</v>
       </c>
       <c r="C97" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D97" t="s">
         <v>71</v>
@@ -8773,7 +8798,7 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="93" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B98" s="93"/>
       <c r="C98" s="93"/>
@@ -8806,7 +8831,7 @@
         <v>24</v>
       </c>
       <c r="C100" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D100" t="s">
         <v>71</v>
@@ -8824,7 +8849,7 @@
         <v>24</v>
       </c>
       <c r="C101" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D101" t="s">
         <v>71</v>
@@ -8842,7 +8867,7 @@
         <v>24</v>
       </c>
       <c r="C102" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D102" t="s">
         <v>71</v>
@@ -8860,7 +8885,7 @@
         <v>24</v>
       </c>
       <c r="C103" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D103" t="s">
         <v>71</v>
@@ -8878,7 +8903,7 @@
         <v>24</v>
       </c>
       <c r="C104" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D104" t="s">
         <v>71</v>
@@ -8896,7 +8921,7 @@
         <v>24</v>
       </c>
       <c r="C105" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D105" t="s">
         <v>71</v>
@@ -8914,7 +8939,7 @@
         <v>24</v>
       </c>
       <c r="C106" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D106" t="s">
         <v>71</v>
@@ -8932,7 +8957,7 @@
         <v>24</v>
       </c>
       <c r="C107" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D107" t="s">
         <v>71</v>
@@ -8950,7 +8975,7 @@
         <v>24</v>
       </c>
       <c r="C108" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D108" t="s">
         <v>71</v>
@@ -8968,7 +8993,7 @@
         <v>24</v>
       </c>
       <c r="C109" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D109" t="s">
         <v>71</v>
@@ -8986,7 +9011,7 @@
         <v>24</v>
       </c>
       <c r="C110" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D110" t="s">
         <v>71</v>
@@ -9004,7 +9029,7 @@
         <v>24</v>
       </c>
       <c r="C111" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D111" t="s">
         <v>71</v>
@@ -9022,7 +9047,7 @@
         <v>24</v>
       </c>
       <c r="C112" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D112" t="s">
         <v>71</v>
@@ -9040,7 +9065,7 @@
         <v>24</v>
       </c>
       <c r="C113" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D113" t="s">
         <v>71</v>
@@ -9058,7 +9083,7 @@
         <v>24</v>
       </c>
       <c r="C114" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D114" t="s">
         <v>71</v>
@@ -9076,7 +9101,7 @@
         <v>24</v>
       </c>
       <c r="C115" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D115" t="s">
         <v>71</v>
@@ -9094,7 +9119,7 @@
         <v>24</v>
       </c>
       <c r="C116" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D116" t="s">
         <v>71</v>
@@ -9130,7 +9155,7 @@
         <v>25</v>
       </c>
       <c r="C118" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D118" t="s">
         <v>71</v>
@@ -9148,7 +9173,7 @@
         <v>25</v>
       </c>
       <c r="C119" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D119" t="s">
         <v>71</v>
@@ -9166,7 +9191,7 @@
         <v>25</v>
       </c>
       <c r="C120" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D120" t="s">
         <v>71</v>
@@ -9184,7 +9209,7 @@
         <v>25</v>
       </c>
       <c r="C121" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D121" t="s">
         <v>71</v>
@@ -9202,7 +9227,7 @@
         <v>25</v>
       </c>
       <c r="C122" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D122" t="s">
         <v>71</v>
@@ -9220,7 +9245,7 @@
         <v>25</v>
       </c>
       <c r="C123" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D123" t="s">
         <v>71</v>
@@ -9238,7 +9263,7 @@
         <v>25</v>
       </c>
       <c r="C124" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D124" t="s">
         <v>71</v>
@@ -9256,7 +9281,7 @@
         <v>25</v>
       </c>
       <c r="C125" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D125" t="s">
         <v>71</v>
@@ -9274,7 +9299,7 @@
         <v>25</v>
       </c>
       <c r="C126" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D126" t="s">
         <v>71</v>
@@ -9292,7 +9317,7 @@
         <v>25</v>
       </c>
       <c r="C127" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D127" t="s">
         <v>71</v>
@@ -9310,7 +9335,7 @@
         <v>25</v>
       </c>
       <c r="C128" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D128" t="s">
         <v>71</v>
@@ -9328,7 +9353,7 @@
         <v>25</v>
       </c>
       <c r="C129" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D129" t="s">
         <v>71</v>
@@ -9346,7 +9371,7 @@
         <v>25</v>
       </c>
       <c r="C130" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D130" t="s">
         <v>71</v>
@@ -9364,7 +9389,7 @@
         <v>25</v>
       </c>
       <c r="C131" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D131" t="s">
         <v>71</v>
@@ -9382,7 +9407,7 @@
         <v>25</v>
       </c>
       <c r="C132" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D132" t="s">
         <v>71</v>
@@ -9400,7 +9425,7 @@
         <v>25</v>
       </c>
       <c r="C133" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D133" t="s">
         <v>71</v>
@@ -9418,7 +9443,7 @@
         <v>25</v>
       </c>
       <c r="C134" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D134" t="s">
         <v>71</v>
@@ -9433,6 +9458,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9457,15 +9483,15 @@
   <sheetData>
     <row r="5" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="90" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C6" s="104" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="105" t="s">
         <v>167</v>
-      </c>
-      <c r="D6" s="105" t="s">
-        <v>168</v>
       </c>
       <c r="E6" s="105"/>
       <c r="F6" s="105"/>
@@ -9474,49 +9500,49 @@
       <c r="I6" s="106"/>
       <c r="J6" s="112"/>
       <c r="M6" s="90" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q6" s="90" t="s">
         <v>238</v>
-      </c>
-      <c r="Q6" s="90" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="7" spans="2:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C7" s="114"/>
       <c r="D7" s="127" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E7" s="127" t="s">
         <v>23</v>
       </c>
       <c r="F7" s="127" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G7" s="127" t="s">
         <v>23</v>
       </c>
       <c r="H7" s="127" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I7" s="128" t="s">
         <v>23</v>
       </c>
       <c r="J7" s="135" t="s">
+        <v>208</v>
+      </c>
+      <c r="L7" s="91" t="s">
         <v>209</v>
       </c>
-      <c r="L7" s="91" t="s">
-        <v>210</v>
-      </c>
       <c r="M7" s="125" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N7" s="131" t="s">
         <v>15</v>
       </c>
       <c r="O7" s="126" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P7" s="91"/>
       <c r="Q7" s="125">
@@ -9539,7 +9565,7 @@
         <v>70</v>
       </c>
       <c r="C8" s="109" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D8" s="78">
         <v>517.6</v>
@@ -9600,10 +9626,10 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C9" s="109" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D9" s="78">
         <v>435.3</v>
@@ -9630,7 +9656,7 @@
         <v>86</v>
       </c>
       <c r="L9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M9" s="97">
         <f>D9*($J9/100)</f>
@@ -9664,10 +9690,10 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C10" s="109" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D10" s="78">
         <v>63.2</v>
@@ -9694,7 +9720,7 @@
         <v>86</v>
       </c>
       <c r="L10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M10" s="97">
         <f>D10*($J10/100)+D36*($J36/100)</f>
@@ -9728,10 +9754,10 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C11" s="109" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D11" s="78">
         <v>5.8</v>
@@ -9758,7 +9784,7 @@
         <v>86</v>
       </c>
       <c r="L11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M11" s="97">
         <f t="shared" ref="M11:M21" si="7">D11*($J11/100)</f>
@@ -9792,10 +9818,10 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C12" s="109" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D12" s="78">
         <v>2.9</v>
@@ -9822,7 +9848,7 @@
         <v>86</v>
       </c>
       <c r="L12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M12" s="97">
         <f t="shared" si="7"/>
@@ -9856,10 +9882,10 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C13" s="109" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D13" s="78">
         <v>10.3</v>
@@ -9886,7 +9912,7 @@
         <v>85</v>
       </c>
       <c r="L13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="M13" s="97">
         <f t="shared" si="7"/>
@@ -9920,10 +9946,10 @@
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C14" s="109" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D14" s="78">
         <v>1.3</v>
@@ -9950,7 +9976,7 @@
         <v>85</v>
       </c>
       <c r="L14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="M14" s="97">
         <f t="shared" si="7"/>
@@ -9984,10 +10010,10 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C15" s="109" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D15" s="78">
         <v>4.3</v>
@@ -10014,7 +10040,7 @@
         <v>91</v>
       </c>
       <c r="L15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M15" s="97">
         <f t="shared" si="7"/>
@@ -10048,10 +10074,10 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C16" s="109" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D16" s="78">
         <v>1.6</v>
@@ -10078,7 +10104,7 @@
         <v>91</v>
       </c>
       <c r="L16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M16" s="97">
         <f t="shared" si="7"/>
@@ -10112,10 +10138,10 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C17" s="109" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D17" s="78">
         <v>88.6</v>
@@ -10142,7 +10168,7 @@
         <v>88</v>
       </c>
       <c r="L17" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="M17" s="97">
         <f t="shared" si="7"/>
@@ -10176,10 +10202,10 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D18" s="78">
         <v>0</v>
@@ -10206,7 +10232,7 @@
         <v>87</v>
       </c>
       <c r="L18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M18" s="97">
         <f t="shared" si="7"/>
@@ -10240,10 +10266,10 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C19" s="109" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D19" s="78">
         <v>40.700000000000003</v>
@@ -10270,7 +10296,7 @@
         <v>90</v>
       </c>
       <c r="L19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="M19" s="97">
         <f t="shared" si="7"/>
@@ -10304,10 +10330,10 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C20" s="109" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D20" s="78">
         <v>5.5</v>
@@ -10334,7 +10360,7 @@
         <v>91</v>
       </c>
       <c r="L20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M20" s="97">
         <f t="shared" si="7"/>
@@ -10368,10 +10394,10 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C21" s="109" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D21" s="78">
         <v>1.6</v>
@@ -10398,7 +10424,7 @@
         <v>91</v>
       </c>
       <c r="L21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M21" s="97">
         <f t="shared" si="7"/>
@@ -10432,10 +10458,10 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C22" s="109" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D22" s="78">
         <v>39.9</v>
@@ -10462,7 +10488,7 @@
         <v>87</v>
       </c>
       <c r="L22" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="M22" s="97">
         <f>D22*($J22/100)+D39*($J39/100)</f>
@@ -10496,13 +10522,13 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="87" t="s">
+        <v>214</v>
+      </c>
+      <c r="B23" t="s">
         <v>215</v>
       </c>
-      <c r="B23" t="s">
-        <v>216</v>
-      </c>
       <c r="C23" s="109" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D23" s="78">
         <v>29.7</v>
@@ -10529,7 +10555,7 @@
         <v>88</v>
       </c>
       <c r="L23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M23" s="97">
         <f>D23*($J23/100)</f>
@@ -10563,10 +10589,10 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C24" s="109" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D24" s="78">
         <v>1.7</v>
@@ -10593,7 +10619,7 @@
         <v>90</v>
       </c>
       <c r="L24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="M24" s="97">
         <f>D24*($J24/100)</f>
@@ -10627,10 +10653,10 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C25" s="109" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D25" s="78">
         <v>60.4</v>
@@ -10657,7 +10683,7 @@
         <v>11</v>
       </c>
       <c r="L25" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="M25" s="97">
         <f>D25*($J25/100)+D37*($J37/100)</f>
@@ -10691,10 +10717,10 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C26" s="109" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D26" s="78">
         <v>5.2</v>
@@ -10721,7 +10747,7 @@
         <v>76</v>
       </c>
       <c r="L26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M26" s="97">
         <f>D26*($J26/100)</f>
@@ -10755,10 +10781,10 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C27" s="109" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D27" s="78">
         <v>8.6999999999999993</v>
@@ -10785,7 +10811,7 @@
         <v>89</v>
       </c>
       <c r="L27" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M27" s="97">
         <f>D27*($J27/100)</f>
@@ -10819,10 +10845,10 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C28" s="109" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D28" s="78">
         <v>188.4</v>
@@ -10849,7 +10875,7 @@
         <v>6.3</v>
       </c>
       <c r="L28" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M28" s="97">
         <f>D28*($J28/100)+D38*($J38/100)</f>
@@ -10883,10 +10909,10 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C29" s="109" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D29" s="78">
         <v>0</v>
@@ -10913,7 +10939,7 @@
         <v>97</v>
       </c>
       <c r="L29" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="M29" s="97">
         <f>D29*($J29/100)</f>
@@ -10947,10 +10973,10 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C30" s="109" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D30" s="78">
         <v>0</v>
@@ -10977,7 +11003,7 @@
         <v>92</v>
       </c>
       <c r="L30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="M30" s="97">
         <f>D30*($J30/100)</f>
@@ -11011,10 +11037,10 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C31" s="109" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D31" s="78">
         <v>2.2000000000000002</v>
@@ -11041,7 +11067,7 @@
         <v>92</v>
       </c>
       <c r="L31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="M31" s="97">
         <f>D31*($J31/100)</f>
@@ -11075,10 +11101,10 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C32" s="109" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D32" s="78">
         <v>2.2999999999999998</v>
@@ -11105,7 +11131,7 @@
         <v>100</v>
       </c>
       <c r="L32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M32" s="97">
         <f>D32*($J32/100)</f>
@@ -11139,10 +11165,10 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B33" s="87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C33" s="141" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D33" s="142">
         <v>62.6</v>
@@ -11167,7 +11193,7 @@
       </c>
       <c r="J33" s="136"/>
       <c r="L33" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M33" s="101">
         <f>D41*($J41/100)</f>
@@ -11201,10 +11227,10 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B34" s="87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C34" s="141" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D34" s="142">
         <v>5.8</v>
@@ -11239,10 +11265,10 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B35" s="87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C35" s="141" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D35" s="142">
         <v>43.3</v>
@@ -11277,10 +11303,10 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C36" s="109" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D36" s="78">
         <v>0</v>
@@ -11318,10 +11344,10 @@
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="87"/>
       <c r="B37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C37" s="117" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D37" s="118">
         <v>0</v>
@@ -11358,10 +11384,10 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C38" s="109" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D38" s="78">
         <v>0</v>
@@ -11398,10 +11424,10 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C39" s="109" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D39" s="78">
         <v>0</v>
@@ -11438,10 +11464,10 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B40" s="87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C40" s="145" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D40" s="142">
         <v>0</v>
@@ -11478,10 +11504,10 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C41" s="109" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D41" s="78">
         <v>0</v>
@@ -11518,10 +11544,10 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B42" s="87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C42" s="146" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D42" s="147">
         <v>0</v>
@@ -11556,7 +11582,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C43" s="121" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D43" s="77">
         <v>2746.2</v>
@@ -11582,7 +11608,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C44" s="107" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D44" s="112">
         <v>4375.1000000000004</v>
@@ -11598,7 +11624,7 @@
       <c r="I44" s="113"/>
       <c r="J44" s="136"/>
       <c r="L44" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="M44" s="123">
         <f>SUM(M8:M43)</f>
@@ -11632,7 +11658,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C45" s="114" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D45" s="115">
         <f>SUM(D8:D42)</f>
@@ -11659,7 +11685,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C47" s="137" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L47" s="103"/>
       <c r="M47" s="87"/>
@@ -11668,7 +11694,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C48" s="137" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L48" s="103"/>
       <c r="M48" s="87"/>
@@ -11689,7 +11715,7 @@
     </row>
     <row r="51" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C51" s="138" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D51" s="118"/>
       <c r="E51" s="118"/>
@@ -11701,7 +11727,7 @@
     </row>
     <row r="52" spans="3:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="150" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D52" s="151"/>
       <c r="E52" s="151"/>
@@ -14594,4 +14620,19 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add to previous commit
</commit_message>
<xml_diff>
--- a/data/default/PigHerd.xlsx
+++ b/data/default/PigHerd.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="250">
   <si>
     <t>parameter</t>
   </si>
@@ -821,6 +821,15 @@
   <si>
     <t>Landquist et al. 2020</t>
   </si>
+  <si>
+    <t>rapeseed cake</t>
+  </si>
+  <si>
+    <t>rapseed cake in organic rations</t>
+  </si>
+  <si>
+    <t>No inclusion</t>
+  </si>
 </sst>
 </file>
 
@@ -832,7 +841,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -988,6 +997,13 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1321,7 +1337,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="167">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1620,6 +1636,8 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1714,7 +1732,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -1844,7 +1861,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -1878,7 +1894,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -1932,7 +1947,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2062,7 +2076,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2096,7 +2109,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2150,7 +2162,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2373,7 +2384,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2407,7 +2417,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -2421,7 +2430,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2466,7 +2474,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2689,7 +2696,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2723,7 +2729,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
@@ -2737,7 +2742,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2782,7 +2786,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2912,7 +2915,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2946,7 +2948,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2985,7 +2986,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3382,7 +3382,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3749,7 +3748,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4121,7 +4119,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -7251,7 +7248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P134"/>
+  <dimension ref="A1:P139"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -8262,7 +8259,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="65" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
         <v>164</v>
       </c>
@@ -8277,7 +8274,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
         <v>217</v>
       </c>
@@ -8292,7 +8289,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C67" t="s">
         <v>218</v>
       </c>
@@ -8307,7 +8304,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
         <v>162</v>
       </c>
@@ -8322,7 +8319,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="69" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
         <v>163</v>
       </c>
@@ -8337,7 +8334,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="70" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
         <v>235</v>
       </c>
@@ -8352,7 +8349,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
         <v>219</v>
       </c>
@@ -8367,7 +8364,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="72" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>27</v>
+      </c>
       <c r="C72" t="s">
         <v>220</v>
       </c>
@@ -8382,121 +8382,127 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C73" t="s">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="C73" s="150" t="s">
+        <v>247</v>
+      </c>
+      <c r="D73" s="150" t="s">
+        <v>71</v>
+      </c>
+      <c r="E73" s="151">
+        <f>E72</f>
+        <v>3.2865954280882512</v>
+      </c>
+      <c r="F73" s="150" t="s">
+        <v>23</v>
+      </c>
+      <c r="G73" s="150" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C74" t="s">
         <v>216</v>
-      </c>
-      <c r="D73" t="s">
-        <v>71</v>
-      </c>
-      <c r="E73" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C73,'feed rations'!$L$8:$L$43,0),MATCH(B73,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.44906934527932563</v>
-      </c>
-      <c r="F73" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="74" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
-        <v>212</v>
       </c>
       <c r="D74" t="s">
         <v>71</v>
       </c>
       <c r="E74" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C74,'feed rations'!$L$8:$L$43,0),MATCH(B74,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.13063835499034929</v>
+        <v>0.44906934527932563</v>
       </c>
       <c r="F74" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="75" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D75" t="s">
         <v>71</v>
       </c>
       <c r="E75" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C75,'feed rations'!$L$8:$L$43,0),MATCH(B75,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.1145942422939523</v>
+        <v>0.13063835499034929</v>
       </c>
       <c r="F75" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="76" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D76" t="s">
         <v>71</v>
       </c>
       <c r="E76" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C76,'feed rations'!$L$8:$L$43,0),MATCH(B76,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.3450302513926982</v>
+        <v>3.1145942422939523</v>
       </c>
       <c r="F76" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="D77" t="s">
         <v>71</v>
       </c>
       <c r="E77" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C77,'feed rations'!$L$8:$L$43,0),MATCH(B77,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.13727794171375987</v>
+        <v>2.3450302513926982</v>
       </c>
       <c r="F77" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C78" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D78" t="s">
         <v>71</v>
       </c>
       <c r="E78" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C78,'feed rations'!$L$8:$L$43,0),MATCH(B78,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.59612721878837949</v>
+        <v>0.13727794171375987</v>
       </c>
       <c r="F78" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="79" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="D79" t="s">
         <v>71</v>
       </c>
       <c r="E79" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C79,'feed rations'!$L$8:$L$43,0),MATCH(B79,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.35458982068809092</v>
+        <v>0.59612721878837949</v>
       </c>
       <c r="F79" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="80" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D80" t="s">
         <v>71</v>
       </c>
       <c r="E80" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C80,'feed rations'!$L$8:$L$43,0),MATCH(B80,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.69473405404551813</v>
+        <v>0.35458982068809092</v>
       </c>
       <c r="F80" t="s">
         <v>23</v>
@@ -8504,14 +8510,14 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="D81" t="s">
         <v>71</v>
       </c>
       <c r="E81" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C81,'feed rations'!$L$8:$L$43,0),MATCH(B81,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.0649538207770974</v>
+        <v>0.69473405404551813</v>
       </c>
       <c r="F81" t="s">
         <v>23</v>
@@ -8519,62 +8525,59 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D82" t="s">
         <v>71</v>
       </c>
       <c r="E82" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C82,'feed rations'!$L$8:$L$43,0),MATCH(B82,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.18160166929977128</v>
+        <v>1.0649538207770974</v>
       </c>
       <c r="F82" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A83" s="93" t="s">
+      <c r="C83" t="s">
+        <v>223</v>
+      </c>
+      <c r="D83" t="s">
+        <v>71</v>
+      </c>
+      <c r="E83" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C83,'feed rations'!$L$8:$L$43,0),MATCH(B83,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.18160166929977128</v>
+      </c>
+      <c r="F83" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="93" t="s">
         <v>232</v>
       </c>
-      <c r="B83" s="93"/>
-      <c r="C83" s="93"/>
-      <c r="D83" s="94"/>
-      <c r="E83" s="95"/>
-      <c r="F83" s="94"/>
-      <c r="G83" s="94"/>
-      <c r="H83" s="93"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>15</v>
-      </c>
-      <c r="C84" t="s">
-        <v>70</v>
-      </c>
-      <c r="D84" t="s">
-        <v>71</v>
-      </c>
-      <c r="E84" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C84,'feed rations'!$L$8:$L$43,0),MATCH(B84,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>37.344664381805039</v>
-      </c>
-      <c r="F84" t="s">
-        <v>23</v>
-      </c>
+      <c r="B84" s="93"/>
+      <c r="C84" s="93"/>
+      <c r="D84" s="94"/>
+      <c r="E84" s="95"/>
+      <c r="F84" s="94"/>
+      <c r="G84" s="94"/>
+      <c r="H84" s="93"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>15</v>
       </c>
       <c r="C85" t="s">
-        <v>159</v>
+        <v>70</v>
       </c>
       <c r="D85" t="s">
         <v>71</v>
       </c>
       <c r="E85" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C85,'feed rations'!$L$8:$L$43,0),MATCH(B85,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>33.835769741903896</v>
+        <v>37.344664381805039</v>
       </c>
       <c r="F85" t="s">
         <v>23</v>
@@ -8585,14 +8588,14 @@
         <v>15</v>
       </c>
       <c r="C86" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D86" t="s">
         <v>71</v>
       </c>
       <c r="E86" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C86,'feed rations'!$L$8:$L$43,0),MATCH(B86,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.2684246112238</v>
+        <v>33.835769741903896</v>
       </c>
       <c r="F86" t="s">
         <v>23</v>
@@ -8603,14 +8606,14 @@
         <v>15</v>
       </c>
       <c r="C87" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D87" t="s">
         <v>71</v>
       </c>
       <c r="E87" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C87,'feed rations'!$L$8:$L$43,0),MATCH(B87,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.7544473199505721</v>
+        <v>7.2684246112238</v>
       </c>
       <c r="F87" t="s">
         <v>23</v>
@@ -8621,14 +8624,14 @@
         <v>15</v>
       </c>
       <c r="C88" t="s">
-        <v>217</v>
+        <v>164</v>
       </c>
       <c r="D88" t="s">
         <v>71</v>
       </c>
       <c r="E88" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C88,'feed rations'!$L$8:$L$43,0),MATCH(B88,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.24772096710265556</v>
+        <v>1.7544473199505721</v>
       </c>
       <c r="F88" t="s">
         <v>23</v>
@@ -8639,14 +8642,14 @@
         <v>15</v>
       </c>
       <c r="C89" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D89" t="s">
         <v>71</v>
       </c>
       <c r="E89" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C89,'feed rations'!$L$8:$L$43,0),MATCH(B89,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.74316290130796658</v>
+        <v>0.24772096710265556</v>
       </c>
       <c r="F89" t="s">
         <v>23</v>
@@ -8657,14 +8660,14 @@
         <v>15</v>
       </c>
       <c r="C90" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="D90" t="s">
         <v>71</v>
       </c>
       <c r="E90" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C90,'feed rations'!$L$8:$L$43,0),MATCH(B90,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.4571821594273857</v>
+        <v>0.74316290130796658</v>
       </c>
       <c r="F90" t="s">
         <v>23</v>
@@ -8675,14 +8678,14 @@
         <v>15</v>
       </c>
       <c r="C91" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="D91" t="s">
         <v>71</v>
       </c>
       <c r="E91" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C91,'feed rations'!$L$8:$L$43,0),MATCH(B91,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.1809936816581557</v>
+        <v>1.4571821594273857</v>
       </c>
       <c r="F91" t="s">
         <v>23</v>
@@ -8693,14 +8696,14 @@
         <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D92" t="s">
         <v>71</v>
       </c>
       <c r="E92" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C92,'feed rations'!$L$8:$L$43,0),MATCH(B92,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.2819472616632859</v>
+        <v>7.1809936816581557</v>
       </c>
       <c r="F92" t="s">
         <v>23</v>
@@ -8711,53 +8714,65 @@
         <v>15</v>
       </c>
       <c r="C93" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D93" t="s">
         <v>71</v>
       </c>
       <c r="E93" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C93,'feed rations'!$L$8:$L$43,0),MATCH(B93,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.2823203002960992</v>
+        <v>2.2819472616632859</v>
       </c>
       <c r="F93" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>27</v>
+      </c>
       <c r="B94" t="s">
         <v>15</v>
       </c>
       <c r="C94" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="D94" t="s">
         <v>71</v>
       </c>
       <c r="E94" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C94,'feed rations'!$L$8:$L$43,0),MATCH(B94,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.7626075400433656</v>
+        <v>0</v>
       </c>
       <c r="F94" t="s">
         <v>23</v>
       </c>
+      <c r="G94" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="150" t="s">
+        <v>28</v>
+      </c>
       <c r="B95" t="s">
         <v>15</v>
       </c>
-      <c r="C95" t="s">
-        <v>230</v>
-      </c>
-      <c r="D95" t="s">
+      <c r="C95" s="150" t="s">
+        <v>247</v>
+      </c>
+      <c r="D95" s="150" t="s">
         <v>71</v>
       </c>
-      <c r="E95" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C95,'feed rations'!$L$8:$L$43,0),MATCH(B95,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.2826933389289128</v>
-      </c>
-      <c r="F95" t="s">
+      <c r="E95" s="151">
+        <f>E94</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="150" t="s">
         <v>23</v>
+      </c>
+      <c r="G95" s="150" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
@@ -8765,14 +8780,14 @@
         <v>15</v>
       </c>
       <c r="C96" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D96" t="s">
         <v>71</v>
       </c>
       <c r="E96" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C96,'feed rations'!$L$8:$L$43,0),MATCH(B96,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.3406075866731948</v>
+        <v>1.2823203002960992</v>
       </c>
       <c r="F96" t="s">
         <v>23</v>
@@ -8783,44 +8798,50 @@
         <v>15</v>
       </c>
       <c r="C97" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D97" t="s">
         <v>71</v>
       </c>
       <c r="E97" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C97,'feed rations'!$L$8:$L$43,0),MATCH(B97,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.2174582080156675</v>
+        <v>1.7626075400433656</v>
       </c>
       <c r="F97" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A98" s="93" t="s">
-        <v>233</v>
-      </c>
-      <c r="B98" s="93"/>
-      <c r="C98" s="93"/>
-      <c r="D98" s="94"/>
-      <c r="E98" s="95"/>
-      <c r="F98" s="94"/>
-      <c r="G98" s="94"/>
-      <c r="H98" s="93"/>
+      <c r="B98" t="s">
+        <v>15</v>
+      </c>
+      <c r="C98" t="s">
+        <v>230</v>
+      </c>
+      <c r="D98" t="s">
+        <v>71</v>
+      </c>
+      <c r="E98" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C98,'feed rations'!$L$8:$L$43,0),MATCH(B98,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.2826933389289128</v>
+      </c>
+      <c r="F98" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C99" t="s">
-        <v>70</v>
+        <v>222</v>
       </c>
       <c r="D99" t="s">
         <v>71</v>
       </c>
       <c r="E99" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C99,'feed rations'!$L$8:$L$43,0),MATCH(B99,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>31.302145183860713</v>
+        <v>1.3406075866731948</v>
       </c>
       <c r="F99" t="s">
         <v>23</v>
@@ -8828,53 +8849,47 @@
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C100" t="s">
-        <v>159</v>
+        <v>223</v>
       </c>
       <c r="D100" t="s">
         <v>71</v>
       </c>
       <c r="E100" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C100,'feed rations'!$L$8:$L$43,0),MATCH(B100,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>24.045914241116183</v>
+        <v>3.2174582080156675</v>
       </c>
       <c r="F100" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B101" t="s">
-        <v>24</v>
-      </c>
-      <c r="C101" t="s">
-        <v>160</v>
-      </c>
-      <c r="D101" t="s">
-        <v>71</v>
-      </c>
-      <c r="E101" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C101,'feed rations'!$L$8:$L$43,0),MATCH(B101,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.0526821754690197</v>
-      </c>
-      <c r="F101" t="s">
-        <v>23</v>
-      </c>
+      <c r="A101" s="93" t="s">
+        <v>233</v>
+      </c>
+      <c r="B101" s="93"/>
+      <c r="C101" s="93"/>
+      <c r="D101" s="94"/>
+      <c r="E101" s="95"/>
+      <c r="F101" s="94"/>
+      <c r="G101" s="94"/>
+      <c r="H101" s="93"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>24</v>
       </c>
       <c r="C102" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="D102" t="s">
         <v>71</v>
       </c>
       <c r="E102" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C102,'feed rations'!$L$8:$L$43,0),MATCH(B102,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.7825033637710859</v>
+        <v>31.302145183860713</v>
       </c>
       <c r="F102" t="s">
         <v>23</v>
@@ -8885,14 +8900,14 @@
         <v>24</v>
       </c>
       <c r="C103" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D103" t="s">
         <v>71</v>
       </c>
       <c r="E103" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C103,'feed rations'!$L$8:$L$43,0),MATCH(B103,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.7193946199409905E-2</v>
+        <v>24.045914241116183</v>
       </c>
       <c r="F103" t="s">
         <v>23</v>
@@ -8903,14 +8918,14 @@
         <v>24</v>
       </c>
       <c r="C104" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="D104" t="s">
         <v>71</v>
       </c>
       <c r="E104" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C104,'feed rations'!$L$8:$L$43,0),MATCH(B104,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.45777805304301217</v>
+        <v>4.0526821754690197</v>
       </c>
       <c r="F104" t="s">
         <v>23</v>
@@ -8921,14 +8936,14 @@
         <v>24</v>
       </c>
       <c r="C105" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="D105" t="s">
         <v>71</v>
       </c>
       <c r="E105" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C105,'feed rations'!$L$8:$L$43,0),MATCH(B105,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.74407873064429</v>
+        <v>3.7825033637710859</v>
       </c>
       <c r="F105" t="s">
         <v>23</v>
@@ -8939,14 +8954,14 @@
         <v>24</v>
       </c>
       <c r="C106" t="s">
-        <v>219</v>
+        <v>164</v>
       </c>
       <c r="D106" t="s">
         <v>71</v>
       </c>
       <c r="E106" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C106,'feed rations'!$L$8:$L$43,0),MATCH(B106,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.8436095530201233</v>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="F106" t="s">
         <v>23</v>
@@ -8957,14 +8972,14 @@
         <v>24</v>
       </c>
       <c r="C107" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D107" t="s">
         <v>71</v>
       </c>
       <c r="E107" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C107,'feed rations'!$L$8:$L$43,0),MATCH(B107,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.5141197601242991</v>
+        <v>0.45777805304301217</v>
       </c>
       <c r="F107" t="s">
         <v>23</v>
@@ -8975,14 +8990,14 @@
         <v>24</v>
       </c>
       <c r="C108" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D108" t="s">
         <v>71</v>
       </c>
       <c r="E108" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C108,'feed rations'!$L$8:$L$43,0),MATCH(B108,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.16336393265456514</v>
+        <v>7.74407873064429</v>
       </c>
       <c r="F108" t="s">
         <v>23</v>
@@ -8993,53 +9008,62 @@
         <v>24</v>
       </c>
       <c r="C109" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D109" t="s">
         <v>71</v>
       </c>
       <c r="E109" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C109,'feed rations'!$L$8:$L$43,0),MATCH(B109,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>8.277704323848349</v>
+        <v>2.8436095530201233</v>
       </c>
       <c r="F109" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>27</v>
+      </c>
       <c r="B110" t="s">
         <v>24</v>
       </c>
       <c r="C110" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D110" t="s">
         <v>71</v>
       </c>
       <c r="E110" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C110,'feed rations'!$L$8:$L$43,0),MATCH(B110,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.86888069675614876</v>
+        <v>3.5141197601242991</v>
       </c>
       <c r="F110" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B111" t="s">
+      <c r="A111" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="B111" s="150" t="s">
         <v>24</v>
       </c>
-      <c r="C111" t="s">
-        <v>224</v>
-      </c>
-      <c r="D111" t="s">
+      <c r="C111" s="150" t="s">
+        <v>247</v>
+      </c>
+      <c r="D111" s="150" t="s">
         <v>71</v>
       </c>
-      <c r="E111" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C111,'feed rations'!$L$8:$L$43,0),MATCH(B111,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.16156872460341609</v>
-      </c>
-      <c r="F111" t="s">
+      <c r="E111" s="151">
+        <f>E110</f>
+        <v>3.5141197601242991</v>
+      </c>
+      <c r="F111" s="150" t="s">
         <v>23</v>
+      </c>
+      <c r="G111" s="150" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -9047,14 +9071,14 @@
         <v>24</v>
       </c>
       <c r="C112" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="D112" t="s">
         <v>71</v>
       </c>
       <c r="E112" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C112,'feed rations'!$L$8:$L$43,0),MATCH(B112,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.6933021685215648</v>
+        <v>0.16336393265456514</v>
       </c>
       <c r="F112" t="s">
         <v>23</v>
@@ -9065,14 +9089,14 @@
         <v>24</v>
       </c>
       <c r="C113" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="D113" t="s">
         <v>71</v>
       </c>
       <c r="E113" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C113,'feed rations'!$L$8:$L$43,0),MATCH(B113,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.554511941275154</v>
+        <v>8.277704323848349</v>
       </c>
       <c r="F113" t="s">
         <v>23</v>
@@ -9083,14 +9107,14 @@
         <v>24</v>
       </c>
       <c r="C114" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D114" t="s">
         <v>71</v>
       </c>
       <c r="E114" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C114,'feed rations'!$L$8:$L$43,0),MATCH(B114,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.10232685891549684</v>
+        <v>0.86888069675614876</v>
       </c>
       <c r="F114" t="s">
         <v>23</v>
@@ -9101,14 +9125,14 @@
         <v>24</v>
       </c>
       <c r="C115" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D115" t="s">
         <v>71</v>
       </c>
       <c r="E115" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C115,'feed rations'!$L$8:$L$43,0),MATCH(B115,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.3583163461771495</v>
+        <v>0.16156872460341609</v>
       </c>
       <c r="F115" t="s">
         <v>23</v>
@@ -9119,14 +9143,14 @@
         <v>24</v>
       </c>
       <c r="C116" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D116" t="s">
         <v>71</v>
       </c>
       <c r="E116" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C116,'feed rations'!$L$8:$L$43,0),MATCH(B116,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0</v>
+        <v>4.6933021685215648</v>
       </c>
       <c r="F116" t="s">
         <v>23</v>
@@ -9134,17 +9158,17 @@
     </row>
     <row r="117" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C117" t="s">
-        <v>70</v>
+        <v>228</v>
       </c>
       <c r="D117" t="s">
         <v>71</v>
       </c>
       <c r="E117" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C117,'feed rations'!$L$8:$L$43,0),MATCH(B117,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>31.302145183860713</v>
+        <v>3.554511941275154</v>
       </c>
       <c r="F117" t="s">
         <v>23</v>
@@ -9152,17 +9176,17 @@
     </row>
     <row r="118" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C118" t="s">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="D118" t="s">
         <v>71</v>
       </c>
       <c r="E118" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C118,'feed rations'!$L$8:$L$43,0),MATCH(B118,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>24.045914241116183</v>
+        <v>0.10232685891549684</v>
       </c>
       <c r="F118" t="s">
         <v>23</v>
@@ -9170,17 +9194,17 @@
     </row>
     <row r="119" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B119" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C119" t="s">
-        <v>160</v>
+        <v>226</v>
       </c>
       <c r="D119" t="s">
         <v>71</v>
       </c>
       <c r="E119" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C119,'feed rations'!$L$8:$L$43,0),MATCH(B119,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.0526821754690197</v>
+        <v>4.3583163461771495</v>
       </c>
       <c r="F119" t="s">
         <v>23</v>
@@ -9188,17 +9212,17 @@
     </row>
     <row r="120" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C120" t="s">
-        <v>161</v>
+        <v>222</v>
       </c>
       <c r="D120" t="s">
         <v>71</v>
       </c>
       <c r="E120" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C120,'feed rations'!$L$8:$L$43,0),MATCH(B120,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.7825033637710859</v>
+        <v>0</v>
       </c>
       <c r="F120" t="s">
         <v>23</v>
@@ -9209,14 +9233,14 @@
         <v>25</v>
       </c>
       <c r="C121" t="s">
-        <v>164</v>
+        <v>70</v>
       </c>
       <c r="D121" t="s">
         <v>71</v>
       </c>
       <c r="E121" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C121,'feed rations'!$L$8:$L$43,0),MATCH(B121,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.7193946199409905E-2</v>
+        <v>31.302145183860713</v>
       </c>
       <c r="F121" t="s">
         <v>23</v>
@@ -9227,14 +9251,14 @@
         <v>25</v>
       </c>
       <c r="C122" t="s">
-        <v>217</v>
+        <v>159</v>
       </c>
       <c r="D122" t="s">
         <v>71</v>
       </c>
       <c r="E122" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C122,'feed rations'!$L$8:$L$43,0),MATCH(B122,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.45777805304301217</v>
+        <v>24.045914241116183</v>
       </c>
       <c r="F122" t="s">
         <v>23</v>
@@ -9245,14 +9269,14 @@
         <v>25</v>
       </c>
       <c r="C123" t="s">
-        <v>218</v>
+        <v>160</v>
       </c>
       <c r="D123" t="s">
         <v>71</v>
       </c>
       <c r="E123" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C123,'feed rations'!$L$8:$L$43,0),MATCH(B123,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.74407873064429</v>
+        <v>4.0526821754690197</v>
       </c>
       <c r="F123" t="s">
         <v>23</v>
@@ -9263,14 +9287,14 @@
         <v>25</v>
       </c>
       <c r="C124" t="s">
-        <v>219</v>
+        <v>161</v>
       </c>
       <c r="D124" t="s">
         <v>71</v>
       </c>
       <c r="E124" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C124,'feed rations'!$L$8:$L$43,0),MATCH(B124,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.8436095530201233</v>
+        <v>3.7825033637710859</v>
       </c>
       <c r="F124" t="s">
         <v>23</v>
@@ -9281,14 +9305,14 @@
         <v>25</v>
       </c>
       <c r="C125" t="s">
-        <v>220</v>
+        <v>164</v>
       </c>
       <c r="D125" t="s">
         <v>71</v>
       </c>
       <c r="E125" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C125,'feed rations'!$L$8:$L$43,0),MATCH(B125,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.5141197601242991</v>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="F125" t="s">
         <v>23</v>
@@ -9299,14 +9323,14 @@
         <v>25</v>
       </c>
       <c r="C126" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D126" t="s">
         <v>71</v>
       </c>
       <c r="E126" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C126,'feed rations'!$L$8:$L$43,0),MATCH(B126,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.16336393265456514</v>
+        <v>0.45777805304301217</v>
       </c>
       <c r="F126" t="s">
         <v>23</v>
@@ -9317,14 +9341,14 @@
         <v>25</v>
       </c>
       <c r="C127" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D127" t="s">
         <v>71</v>
       </c>
       <c r="E127" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C127,'feed rations'!$L$8:$L$43,0),MATCH(B127,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>8.277704323848349</v>
+        <v>7.74407873064429</v>
       </c>
       <c r="F127" t="s">
         <v>23</v>
@@ -9335,124 +9359,223 @@
         <v>25</v>
       </c>
       <c r="C128" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D128" t="s">
         <v>71</v>
       </c>
       <c r="E128" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C128,'feed rations'!$L$8:$L$43,0),MATCH(B128,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.86888069675614876</v>
+        <v>2.8436095530201233</v>
       </c>
       <c r="F128" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>27</v>
+      </c>
       <c r="B129" t="s">
         <v>25</v>
       </c>
       <c r="C129" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D129" t="s">
         <v>71</v>
       </c>
       <c r="E129" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C129,'feed rations'!$L$8:$L$43,0),MATCH(B129,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.16156872460341609</v>
+        <v>3.5141197601242991</v>
       </c>
       <c r="F129" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B130" t="s">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A130" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="B130" s="150" t="s">
         <v>25</v>
       </c>
-      <c r="C130" t="s">
-        <v>225</v>
-      </c>
-      <c r="D130" t="s">
+      <c r="C130" s="150" t="s">
+        <v>247</v>
+      </c>
+      <c r="D130" s="150" t="s">
         <v>71</v>
       </c>
-      <c r="E130" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C130,'feed rations'!$L$8:$L$43,0),MATCH(B130,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.6933021685215648</v>
-      </c>
-      <c r="F130" t="s">
+      <c r="E130" s="151">
+        <f>E129</f>
+        <v>3.5141197601242991</v>
+      </c>
+      <c r="F130" s="150" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G130" s="150" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
         <v>25</v>
       </c>
       <c r="C131" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="D131" t="s">
         <v>71</v>
       </c>
       <c r="E131" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C131,'feed rations'!$L$8:$L$43,0),MATCH(B131,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>3.554511941275154</v>
+        <v>0.16336393265456514</v>
       </c>
       <c r="F131" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
         <v>25</v>
       </c>
       <c r="C132" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D132" t="s">
         <v>71</v>
       </c>
       <c r="E132" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C132,'feed rations'!$L$8:$L$43,0),MATCH(B132,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.10232685891549684</v>
+        <v>8.277704323848349</v>
       </c>
       <c r="F132" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>25</v>
       </c>
       <c r="C133" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="D133" t="s">
         <v>71</v>
       </c>
       <c r="E133" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C133,'feed rations'!$L$8:$L$43,0),MATCH(B133,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>4.3583163461771495</v>
+        <v>0.86888069675614876</v>
       </c>
       <c r="F133" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>25</v>
       </c>
       <c r="C134" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D134" t="s">
         <v>71</v>
       </c>
       <c r="E134" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C134,'feed rations'!$L$8:$L$43,0),MATCH(B134,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0</v>
+        <v>0.16156872460341609</v>
       </c>
       <c r="F134" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>25</v>
+      </c>
+      <c r="C135" t="s">
+        <v>225</v>
+      </c>
+      <c r="D135" t="s">
+        <v>71</v>
+      </c>
+      <c r="E135" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C135,'feed rations'!$L$8:$L$43,0),MATCH(B135,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.6933021685215648</v>
+      </c>
+      <c r="F135" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>25</v>
+      </c>
+      <c r="C136" t="s">
+        <v>228</v>
+      </c>
+      <c r="D136" t="s">
+        <v>71</v>
+      </c>
+      <c r="E136" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C136,'feed rations'!$L$8:$L$43,0),MATCH(B136,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.554511941275154</v>
+      </c>
+      <c r="F136" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>25</v>
+      </c>
+      <c r="C137" t="s">
+        <v>210</v>
+      </c>
+      <c r="D137" t="s">
+        <v>71</v>
+      </c>
+      <c r="E137" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C137,'feed rations'!$L$8:$L$43,0),MATCH(B137,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.10232685891549684</v>
+      </c>
+      <c r="F137" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>25</v>
+      </c>
+      <c r="C138" t="s">
+        <v>226</v>
+      </c>
+      <c r="D138" t="s">
+        <v>71</v>
+      </c>
+      <c r="E138" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C138,'feed rations'!$L$8:$L$43,0),MATCH(B138,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.3583163461771495</v>
+      </c>
+      <c r="F138" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>25</v>
+      </c>
+      <c r="C139" t="s">
+        <v>222</v>
+      </c>
+      <c r="D139" t="s">
+        <v>71</v>
+      </c>
+      <c r="E139" s="62">
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C139,'feed rations'!$L$8:$L$43,0),MATCH(B139,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F139" t="s">
         <v>23</v>
       </c>
     </row>
@@ -11726,15 +11849,15 @@
       <c r="J51" s="78"/>
     </row>
     <row r="52" spans="3:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="150" t="s">
+      <c r="C52" s="152" t="s">
         <v>243</v>
       </c>
-      <c r="D52" s="151"/>
-      <c r="E52" s="151"/>
-      <c r="F52" s="151"/>
-      <c r="G52" s="151"/>
-      <c r="H52" s="151"/>
-      <c r="I52" s="152"/>
+      <c r="D52" s="153"/>
+      <c r="E52" s="153"/>
+      <c r="F52" s="153"/>
+      <c r="G52" s="153"/>
+      <c r="H52" s="153"/>
+      <c r="I52" s="154"/>
       <c r="J52" s="140"/>
     </row>
   </sheetData>
@@ -13994,19 +14117,19 @@
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="40"/>
-      <c r="C23" s="159" t="s">
+      <c r="C23" s="161" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="161" t="s">
+      <c r="D23" s="163" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="154" t="s">
+      <c r="E23" s="156" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="156" t="s">
+      <c r="F23" s="158" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="158"/>
+      <c r="G23" s="160"/>
       <c r="H23" s="31"/>
       <c r="O23">
         <v>11</v>
@@ -14028,11 +14151,11 @@
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" s="41"/>
-      <c r="C24" s="160"/>
-      <c r="D24" s="162"/>
-      <c r="E24" s="155"/>
-      <c r="F24" s="157"/>
-      <c r="G24" s="158"/>
+      <c r="C24" s="162"/>
+      <c r="D24" s="164"/>
+      <c r="E24" s="157"/>
+      <c r="F24" s="159"/>
+      <c r="G24" s="160"/>
       <c r="H24" s="18"/>
       <c r="O24">
         <v>13</v>
@@ -14053,13 +14176,13 @@
       </c>
     </row>
     <row r="25" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="164" t="s">
+      <c r="B25" s="166" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="164"/>
-      <c r="D25" s="164"/>
-      <c r="E25" s="164"/>
-      <c r="F25" s="164"/>
+      <c r="C25" s="166"/>
+      <c r="D25" s="166"/>
+      <c r="E25" s="166"/>
+      <c r="F25" s="166"/>
       <c r="G25" s="42"/>
       <c r="H25" s="18"/>
       <c r="O25">
@@ -14081,13 +14204,13 @@
       </c>
     </row>
     <row r="26" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="153" t="s">
+      <c r="B26" s="155" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="153"/>
-      <c r="D26" s="153"/>
-      <c r="E26" s="153"/>
-      <c r="F26" s="153"/>
+      <c r="C26" s="155"/>
+      <c r="D26" s="155"/>
+      <c r="E26" s="155"/>
+      <c r="F26" s="155"/>
       <c r="G26" s="42"/>
       <c r="H26" s="18"/>
       <c r="O26">
@@ -14279,25 +14402,25 @@
       <c r="R33" s="3"/>
     </row>
     <row r="34" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="163" t="s">
+      <c r="B34" s="165" t="s">
         <v>8</v>
       </c>
-      <c r="C34" s="163"/>
-      <c r="D34" s="163"/>
-      <c r="E34" s="163"/>
-      <c r="F34" s="163"/>
+      <c r="C34" s="165"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="165"/>
+      <c r="F34" s="165"/>
       <c r="G34" s="42"/>
       <c r="H34" s="18"/>
       <c r="R34" s="13"/>
     </row>
     <row r="35" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="153" t="s">
+      <c r="B35" s="155" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="153"/>
-      <c r="D35" s="153"/>
-      <c r="E35" s="153"/>
-      <c r="F35" s="153"/>
+      <c r="C35" s="155"/>
+      <c r="D35" s="155"/>
+      <c r="E35" s="155"/>
+      <c r="F35" s="155"/>
       <c r="G35" s="42"/>
       <c r="H35" s="18"/>
     </row>

</xml_diff>

<commit_message>
Name change 'recruitment' -> 'replacement' + data updates after com. w. Mikaela L and Anna H
</commit_message>
<xml_diff>
--- a/data/default/PigHerd.xlsx
+++ b/data/default/PigHerd.xlsx
@@ -147,9 +147,6 @@
   </si>
   <si>
     <t>age_at_first_farrowing</t>
-  </si>
-  <si>
-    <t>recruitment_rate</t>
   </si>
   <si>
     <t>Slakt</t>
@@ -829,6 +826,9 @@
   </si>
   <si>
     <t>No inclusion</t>
+  </si>
+  <si>
+    <t>replacement_rate</t>
   </si>
 </sst>
 </file>
@@ -7261,13 +7261,13 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -7287,7 +7287,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -7312,7 +7312,7 @@
         <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -7330,7 +7330,7 @@
         <v>31</v>
       </c>
       <c r="H4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -7348,7 +7348,7 @@
         <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -7366,7 +7366,7 @@
         <v>31</v>
       </c>
       <c r="H6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -7384,7 +7384,7 @@
         <v>31</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -7402,7 +7402,7 @@
         <v>31</v>
       </c>
       <c r="G8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -7444,7 +7444,7 @@
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>249</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -7464,7 +7464,7 @@
         <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>249</v>
       </c>
       <c r="E12">
         <v>40</v>
@@ -7482,7 +7482,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E13" s="13">
         <v>115</v>
@@ -7494,7 +7494,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E14">
         <v>1.0999999999999999E-2</v>
@@ -7511,7 +7511,7 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -7523,48 +7523,48 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17">
         <v>1.5</v>
       </c>
       <c r="F17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="15" t="s">
         <v>77</v>
-      </c>
-      <c r="H17" s="15" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E18">
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E19">
         <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -7572,17 +7572,17 @@
         <v>13</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E20" s="13">
         <f>E45/0.75</f>
         <v>240.64979221760481</v>
       </c>
       <c r="F20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H20" s="15"/>
     </row>
@@ -7591,39 +7591,39 @@
         <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E21" s="13">
         <f t="shared" ref="E21:E22" si="0">E46/0.75</f>
         <v>205.63847429519072</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H21" s="15"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E22" s="13">
         <f t="shared" si="0"/>
         <v>122.41258802745277</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H22" s="15"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -7772,7 +7772,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -7797,7 +7797,7 @@
         <v>23</v>
       </c>
       <c r="H34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N34" s="62"/>
     </row>
@@ -7816,7 +7816,7 @@
         <v>23</v>
       </c>
       <c r="H35" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -7834,7 +7834,7 @@
         <v>23</v>
       </c>
       <c r="H36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M36" s="13"/>
     </row>
@@ -7853,7 +7853,7 @@
         <v>23</v>
       </c>
       <c r="H37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -7958,7 +7958,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -7973,16 +7973,16 @@
         <v>13</v>
       </c>
       <c r="D45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E45" s="13">
         <v>180.4873441632036</v>
       </c>
       <c r="F45" t="s">
+        <v>66</v>
+      </c>
+      <c r="H45" t="s">
         <v>67</v>
-      </c>
-      <c r="H45" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -7990,16 +7990,16 @@
         <v>14</v>
       </c>
       <c r="D46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E46" s="13">
         <v>154.22885572139305</v>
       </c>
       <c r="F46" t="s">
+        <v>66</v>
+      </c>
+      <c r="H46" t="s">
         <v>67</v>
-      </c>
-      <c r="H46" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -8007,33 +8007,33 @@
         <v>25</v>
       </c>
       <c r="D47" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E47" s="13">
         <v>91.809441020589574</v>
       </c>
       <c r="F47" t="s">
+        <v>66</v>
+      </c>
+      <c r="H47" t="s">
         <v>67</v>
-      </c>
-      <c r="H47" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D48" s="88" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E48" s="89">
         <v>0</v>
       </c>
       <c r="F48" s="88"/>
       <c r="G48" s="88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -8048,19 +8048,19 @@
         <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E50" s="3">
         <v>19.5</v>
       </c>
       <c r="F50" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -8068,20 +8068,20 @@
         <v>24</v>
       </c>
       <c r="D51" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E51" s="3">
         <f>AVERAGE(26.4,25.7,25.4,25.8,25.3)</f>
         <v>25.72</v>
       </c>
       <c r="F51" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G51" s="87" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -8089,20 +8089,20 @@
         <v>25</v>
       </c>
       <c r="D52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E52" s="3">
         <f>AVERAGE(26.4,25.7,25.4,25.8,25.3)</f>
         <v>25.72</v>
       </c>
       <c r="F52" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G52" s="87" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H52" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -8110,7 +8110,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -8118,22 +8118,22 @@
       <c r="E54" s="8"/>
       <c r="F54" s="8"/>
       <c r="G54" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D55" s="88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E55" s="88">
         <v>0</v>
       </c>
       <c r="F55" s="88"/>
       <c r="G55" s="88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -8141,14 +8141,14 @@
         <v>15</v>
       </c>
       <c r="D56" s="88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E56" s="96">
         <v>0</v>
       </c>
       <c r="F56" s="88"/>
       <c r="G56" s="88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -8156,14 +8156,14 @@
         <v>24</v>
       </c>
       <c r="D57" s="88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E57" s="96">
         <v>0</v>
       </c>
       <c r="F57" s="88"/>
       <c r="G57" s="88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -8171,14 +8171,14 @@
         <v>25</v>
       </c>
       <c r="D58" s="88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E58" s="96">
         <v>0</v>
       </c>
       <c r="F58" s="88"/>
       <c r="G58" s="88" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -8189,7 +8189,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="93" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B60" s="93"/>
       <c r="C60" s="93"/>
@@ -8201,10 +8201,10 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C61" t="s">
+        <v>69</v>
+      </c>
+      <c r="D61" t="s">
         <v>70</v>
-      </c>
-      <c r="D61" t="s">
-        <v>71</v>
       </c>
       <c r="E61" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C61,'feed rations'!$L$8:$L$43,0),MATCH(B61,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8216,10 +8216,10 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C62" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E62" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C62,'feed rations'!$L$8:$L$43,0),MATCH(B62,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8231,10 +8231,10 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C63" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E63" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C63,'feed rations'!$L$8:$L$43,0),MATCH(B63,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8246,10 +8246,10 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C64" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D64" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E64" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C64,'feed rations'!$L$8:$L$43,0),MATCH(B64,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8261,10 +8261,10 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D65" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E65" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C65,'feed rations'!$L$8:$L$43,0),MATCH(B65,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8276,10 +8276,10 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E66" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C66,'feed rations'!$L$8:$L$43,0),MATCH(B66,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8291,10 +8291,10 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C67" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D67" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E67" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C67,'feed rations'!$L$8:$L$43,0),MATCH(B67,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8306,10 +8306,10 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E68" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C68,'feed rations'!$L$8:$L$43,0),MATCH(B68,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8321,10 +8321,10 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E69" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C69,'feed rations'!$L$8:$L$43,0),MATCH(B69,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8336,10 +8336,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E70" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C70,'feed rations'!$L$8:$L$43,0),MATCH(B70,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8351,10 +8351,10 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D71" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E71" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C71,'feed rations'!$L$8:$L$43,0),MATCH(B71,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8369,10 +8369,10 @@
         <v>27</v>
       </c>
       <c r="C72" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E72" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C72,'feed rations'!$L$8:$L$43,0),MATCH(B72,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8387,10 +8387,10 @@
         <v>28</v>
       </c>
       <c r="C73" s="150" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D73" s="150" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E73" s="151">
         <f>E72</f>
@@ -8400,15 +8400,15 @@
         <v>23</v>
       </c>
       <c r="G73" s="150" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C74" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D74" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E74" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C74,'feed rations'!$L$8:$L$43,0),MATCH(B74,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8420,10 +8420,10 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D75" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E75" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C75,'feed rations'!$L$8:$L$43,0),MATCH(B75,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8435,10 +8435,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E76" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C76,'feed rations'!$L$8:$L$43,0),MATCH(B76,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8450,10 +8450,10 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C77" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D77" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E77" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C77,'feed rations'!$L$8:$L$43,0),MATCH(B77,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8465,10 +8465,10 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C78" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D78" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E78" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C78,'feed rations'!$L$8:$L$43,0),MATCH(B78,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8480,10 +8480,10 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D79" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E79" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C79,'feed rations'!$L$8:$L$43,0),MATCH(B79,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8495,10 +8495,10 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D80" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E80" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C80,'feed rations'!$L$8:$L$43,0),MATCH(B80,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8510,10 +8510,10 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D81" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E81" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C81,'feed rations'!$L$8:$L$43,0),MATCH(B81,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8525,10 +8525,10 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D82" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E82" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C82,'feed rations'!$L$8:$L$43,0),MATCH(B82,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8540,10 +8540,10 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C83" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D83" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E83" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C83,'feed rations'!$L$8:$L$43,0),MATCH(B83,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8555,7 +8555,7 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="93" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B84" s="93"/>
       <c r="C84" s="93"/>
@@ -8570,10 +8570,10 @@
         <v>15</v>
       </c>
       <c r="C85" t="s">
+        <v>69</v>
+      </c>
+      <c r="D85" t="s">
         <v>70</v>
-      </c>
-      <c r="D85" t="s">
-        <v>71</v>
       </c>
       <c r="E85" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C85,'feed rations'!$L$8:$L$43,0),MATCH(B85,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8588,10 +8588,10 @@
         <v>15</v>
       </c>
       <c r="C86" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D86" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E86" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C86,'feed rations'!$L$8:$L$43,0),MATCH(B86,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8606,10 +8606,10 @@
         <v>15</v>
       </c>
       <c r="C87" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D87" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E87" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C87,'feed rations'!$L$8:$L$43,0),MATCH(B87,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8624,10 +8624,10 @@
         <v>15</v>
       </c>
       <c r="C88" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E88" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C88,'feed rations'!$L$8:$L$43,0),MATCH(B88,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8642,10 +8642,10 @@
         <v>15</v>
       </c>
       <c r="C89" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D89" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E89" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C89,'feed rations'!$L$8:$L$43,0),MATCH(B89,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8660,10 +8660,10 @@
         <v>15</v>
       </c>
       <c r="C90" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D90" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E90" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C90,'feed rations'!$L$8:$L$43,0),MATCH(B90,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8678,10 +8678,10 @@
         <v>15</v>
       </c>
       <c r="C91" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E91" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C91,'feed rations'!$L$8:$L$43,0),MATCH(B91,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8696,10 +8696,10 @@
         <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D92" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E92" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C92,'feed rations'!$L$8:$L$43,0),MATCH(B92,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8714,10 +8714,10 @@
         <v>15</v>
       </c>
       <c r="C93" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D93" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E93" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C93,'feed rations'!$L$8:$L$43,0),MATCH(B93,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8735,10 +8735,10 @@
         <v>15</v>
       </c>
       <c r="C94" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D94" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E94" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C94,'feed rations'!$L$8:$L$43,0),MATCH(B94,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8748,7 +8748,7 @@
         <v>23</v>
       </c>
       <c r="G94" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -8759,10 +8759,10 @@
         <v>15</v>
       </c>
       <c r="C95" s="150" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D95" s="150" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E95" s="151">
         <f>E94</f>
@@ -8772,7 +8772,7 @@
         <v>23</v>
       </c>
       <c r="G95" s="150" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
@@ -8780,10 +8780,10 @@
         <v>15</v>
       </c>
       <c r="C96" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D96" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E96" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C96,'feed rations'!$L$8:$L$43,0),MATCH(B96,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8798,10 +8798,10 @@
         <v>15</v>
       </c>
       <c r="C97" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D97" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E97" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C97,'feed rations'!$L$8:$L$43,0),MATCH(B97,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8816,10 +8816,10 @@
         <v>15</v>
       </c>
       <c r="C98" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D98" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E98" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C98,'feed rations'!$L$8:$L$43,0),MATCH(B98,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8834,10 +8834,10 @@
         <v>15</v>
       </c>
       <c r="C99" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D99" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E99" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C99,'feed rations'!$L$8:$L$43,0),MATCH(B99,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8852,10 +8852,10 @@
         <v>15</v>
       </c>
       <c r="C100" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D100" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E100" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C100,'feed rations'!$L$8:$L$43,0),MATCH(B100,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8867,7 +8867,7 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="93" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B101" s="93"/>
       <c r="C101" s="93"/>
@@ -8882,10 +8882,10 @@
         <v>24</v>
       </c>
       <c r="C102" t="s">
+        <v>69</v>
+      </c>
+      <c r="D102" t="s">
         <v>70</v>
-      </c>
-      <c r="D102" t="s">
-        <v>71</v>
       </c>
       <c r="E102" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C102,'feed rations'!$L$8:$L$43,0),MATCH(B102,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8900,10 +8900,10 @@
         <v>24</v>
       </c>
       <c r="C103" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D103" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E103" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C103,'feed rations'!$L$8:$L$43,0),MATCH(B103,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8918,10 +8918,10 @@
         <v>24</v>
       </c>
       <c r="C104" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D104" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E104" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C104,'feed rations'!$L$8:$L$43,0),MATCH(B104,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8936,10 +8936,10 @@
         <v>24</v>
       </c>
       <c r="C105" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D105" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E105" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C105,'feed rations'!$L$8:$L$43,0),MATCH(B105,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8954,10 +8954,10 @@
         <v>24</v>
       </c>
       <c r="C106" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D106" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E106" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C106,'feed rations'!$L$8:$L$43,0),MATCH(B106,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8972,10 +8972,10 @@
         <v>24</v>
       </c>
       <c r="C107" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D107" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E107" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C107,'feed rations'!$L$8:$L$43,0),MATCH(B107,'feed rations'!$Q$7:$T$7,0))</f>
@@ -8990,10 +8990,10 @@
         <v>24</v>
       </c>
       <c r="C108" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D108" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E108" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C108,'feed rations'!$L$8:$L$43,0),MATCH(B108,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9008,10 +9008,10 @@
         <v>24</v>
       </c>
       <c r="C109" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D109" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E109" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C109,'feed rations'!$L$8:$L$43,0),MATCH(B109,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9029,10 +9029,10 @@
         <v>24</v>
       </c>
       <c r="C110" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D110" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E110" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C110,'feed rations'!$L$8:$L$43,0),MATCH(B110,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9050,10 +9050,10 @@
         <v>24</v>
       </c>
       <c r="C111" s="150" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D111" s="150" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E111" s="151">
         <f>E110</f>
@@ -9063,7 +9063,7 @@
         <v>23</v>
       </c>
       <c r="G111" s="150" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -9071,10 +9071,10 @@
         <v>24</v>
       </c>
       <c r="C112" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D112" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E112" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C112,'feed rations'!$L$8:$L$43,0),MATCH(B112,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9089,10 +9089,10 @@
         <v>24</v>
       </c>
       <c r="C113" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D113" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E113" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C113,'feed rations'!$L$8:$L$43,0),MATCH(B113,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9107,10 +9107,10 @@
         <v>24</v>
       </c>
       <c r="C114" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D114" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E114" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C114,'feed rations'!$L$8:$L$43,0),MATCH(B114,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9125,10 +9125,10 @@
         <v>24</v>
       </c>
       <c r="C115" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D115" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E115" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C115,'feed rations'!$L$8:$L$43,0),MATCH(B115,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9143,10 +9143,10 @@
         <v>24</v>
       </c>
       <c r="C116" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D116" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E116" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C116,'feed rations'!$L$8:$L$43,0),MATCH(B116,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9161,10 +9161,10 @@
         <v>24</v>
       </c>
       <c r="C117" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D117" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E117" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C117,'feed rations'!$L$8:$L$43,0),MATCH(B117,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9179,10 +9179,10 @@
         <v>24</v>
       </c>
       <c r="C118" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D118" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E118" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C118,'feed rations'!$L$8:$L$43,0),MATCH(B118,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9197,10 +9197,10 @@
         <v>24</v>
       </c>
       <c r="C119" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D119" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E119" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C119,'feed rations'!$L$8:$L$43,0),MATCH(B119,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9215,10 +9215,10 @@
         <v>24</v>
       </c>
       <c r="C120" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D120" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E120" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C120,'feed rations'!$L$8:$L$43,0),MATCH(B120,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9233,10 +9233,10 @@
         <v>25</v>
       </c>
       <c r="C121" t="s">
+        <v>69</v>
+      </c>
+      <c r="D121" t="s">
         <v>70</v>
-      </c>
-      <c r="D121" t="s">
-        <v>71</v>
       </c>
       <c r="E121" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C121,'feed rations'!$L$8:$L$43,0),MATCH(B121,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9251,10 +9251,10 @@
         <v>25</v>
       </c>
       <c r="C122" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D122" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E122" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C122,'feed rations'!$L$8:$L$43,0),MATCH(B122,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9269,10 +9269,10 @@
         <v>25</v>
       </c>
       <c r="C123" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D123" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E123" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C123,'feed rations'!$L$8:$L$43,0),MATCH(B123,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9287,10 +9287,10 @@
         <v>25</v>
       </c>
       <c r="C124" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D124" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E124" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C124,'feed rations'!$L$8:$L$43,0),MATCH(B124,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9305,10 +9305,10 @@
         <v>25</v>
       </c>
       <c r="C125" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D125" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E125" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C125,'feed rations'!$L$8:$L$43,0),MATCH(B125,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9323,10 +9323,10 @@
         <v>25</v>
       </c>
       <c r="C126" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D126" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E126" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C126,'feed rations'!$L$8:$L$43,0),MATCH(B126,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9341,10 +9341,10 @@
         <v>25</v>
       </c>
       <c r="C127" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D127" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E127" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C127,'feed rations'!$L$8:$L$43,0),MATCH(B127,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9359,10 +9359,10 @@
         <v>25</v>
       </c>
       <c r="C128" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D128" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E128" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C128,'feed rations'!$L$8:$L$43,0),MATCH(B128,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9380,10 +9380,10 @@
         <v>25</v>
       </c>
       <c r="C129" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D129" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E129" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C129,'feed rations'!$L$8:$L$43,0),MATCH(B129,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9401,10 +9401,10 @@
         <v>25</v>
       </c>
       <c r="C130" s="150" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D130" s="150" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E130" s="151">
         <f>E129</f>
@@ -9414,7 +9414,7 @@
         <v>23</v>
       </c>
       <c r="G130" s="150" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
@@ -9422,10 +9422,10 @@
         <v>25</v>
       </c>
       <c r="C131" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D131" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E131" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C131,'feed rations'!$L$8:$L$43,0),MATCH(B131,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9440,10 +9440,10 @@
         <v>25</v>
       </c>
       <c r="C132" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D132" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E132" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C132,'feed rations'!$L$8:$L$43,0),MATCH(B132,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9458,10 +9458,10 @@
         <v>25</v>
       </c>
       <c r="C133" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D133" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E133" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C133,'feed rations'!$L$8:$L$43,0),MATCH(B133,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9476,10 +9476,10 @@
         <v>25</v>
       </c>
       <c r="C134" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D134" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E134" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C134,'feed rations'!$L$8:$L$43,0),MATCH(B134,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9494,10 +9494,10 @@
         <v>25</v>
       </c>
       <c r="C135" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D135" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E135" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C135,'feed rations'!$L$8:$L$43,0),MATCH(B135,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9512,10 +9512,10 @@
         <v>25</v>
       </c>
       <c r="C136" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D136" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E136" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C136,'feed rations'!$L$8:$L$43,0),MATCH(B136,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9530,10 +9530,10 @@
         <v>25</v>
       </c>
       <c r="C137" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D137" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E137" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C137,'feed rations'!$L$8:$L$43,0),MATCH(B137,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9548,10 +9548,10 @@
         <v>25</v>
       </c>
       <c r="C138" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D138" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E138" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C138,'feed rations'!$L$8:$L$43,0),MATCH(B138,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9566,10 +9566,10 @@
         <v>25</v>
       </c>
       <c r="C139" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D139" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E139" s="62">
         <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C139,'feed rations'!$L$8:$L$43,0),MATCH(B139,'feed rations'!$Q$7:$T$7,0))</f>
@@ -9606,15 +9606,15 @@
   <sheetData>
     <row r="5" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="90" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C6" s="104" t="s">
+        <v>165</v>
+      </c>
+      <c r="D6" s="105" t="s">
         <v>166</v>
-      </c>
-      <c r="D6" s="105" t="s">
-        <v>167</v>
       </c>
       <c r="E6" s="105"/>
       <c r="F6" s="105"/>
@@ -9623,49 +9623,49 @@
       <c r="I6" s="106"/>
       <c r="J6" s="112"/>
       <c r="M6" s="90" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q6" s="90" t="s">
         <v>237</v>
-      </c>
-      <c r="Q6" s="90" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="7" spans="2:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C7" s="114"/>
       <c r="D7" s="127" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E7" s="127" t="s">
         <v>23</v>
       </c>
       <c r="F7" s="127" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G7" s="127" t="s">
         <v>23</v>
       </c>
       <c r="H7" s="127" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I7" s="128" t="s">
         <v>23</v>
       </c>
       <c r="J7" s="135" t="s">
+        <v>207</v>
+      </c>
+      <c r="L7" s="91" t="s">
         <v>208</v>
       </c>
-      <c r="L7" s="91" t="s">
-        <v>209</v>
-      </c>
       <c r="M7" s="125" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N7" s="131" t="s">
         <v>15</v>
       </c>
       <c r="O7" s="126" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="P7" s="91"/>
       <c r="Q7" s="125">
@@ -9685,10 +9685,10 @@
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" s="109" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D8" s="78">
         <v>517.6</v>
@@ -9715,7 +9715,7 @@
         <v>86</v>
       </c>
       <c r="L8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M8" s="97">
         <f>D8*($J8/100)</f>
@@ -9749,10 +9749,10 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C9" s="109" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D9" s="78">
         <v>435.3</v>
@@ -9779,7 +9779,7 @@
         <v>86</v>
       </c>
       <c r="L9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M9" s="97">
         <f>D9*($J9/100)</f>
@@ -9813,10 +9813,10 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C10" s="109" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D10" s="78">
         <v>63.2</v>
@@ -9843,7 +9843,7 @@
         <v>86</v>
       </c>
       <c r="L10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M10" s="97">
         <f>D10*($J10/100)+D36*($J36/100)</f>
@@ -9877,10 +9877,10 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C11" s="109" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D11" s="78">
         <v>5.8</v>
@@ -9907,7 +9907,7 @@
         <v>86</v>
       </c>
       <c r="L11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M11" s="97">
         <f t="shared" ref="M11:M21" si="7">D11*($J11/100)</f>
@@ -9941,10 +9941,10 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C12" s="109" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D12" s="78">
         <v>2.9</v>
@@ -9971,7 +9971,7 @@
         <v>86</v>
       </c>
       <c r="L12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M12" s="97">
         <f t="shared" si="7"/>
@@ -10005,10 +10005,10 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C13" s="109" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D13" s="78">
         <v>10.3</v>
@@ -10035,7 +10035,7 @@
         <v>85</v>
       </c>
       <c r="L13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M13" s="97">
         <f t="shared" si="7"/>
@@ -10069,10 +10069,10 @@
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C14" s="109" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D14" s="78">
         <v>1.3</v>
@@ -10099,7 +10099,7 @@
         <v>85</v>
       </c>
       <c r="L14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="M14" s="97">
         <f t="shared" si="7"/>
@@ -10133,10 +10133,10 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C15" s="109" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D15" s="78">
         <v>4.3</v>
@@ -10163,7 +10163,7 @@
         <v>91</v>
       </c>
       <c r="L15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M15" s="97">
         <f t="shared" si="7"/>
@@ -10197,10 +10197,10 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C16" s="109" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D16" s="78">
         <v>1.6</v>
@@ -10227,7 +10227,7 @@
         <v>91</v>
       </c>
       <c r="L16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M16" s="97">
         <f t="shared" si="7"/>
@@ -10261,10 +10261,10 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C17" s="109" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D17" s="78">
         <v>88.6</v>
@@ -10291,7 +10291,7 @@
         <v>88</v>
       </c>
       <c r="L17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="M17" s="97">
         <f t="shared" si="7"/>
@@ -10325,10 +10325,10 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C18" s="109" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D18" s="78">
         <v>0</v>
@@ -10355,7 +10355,7 @@
         <v>87</v>
       </c>
       <c r="L18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="M18" s="97">
         <f t="shared" si="7"/>
@@ -10389,10 +10389,10 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C19" s="109" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D19" s="78">
         <v>40.700000000000003</v>
@@ -10419,7 +10419,7 @@
         <v>90</v>
       </c>
       <c r="L19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="M19" s="97">
         <f t="shared" si="7"/>
@@ -10453,10 +10453,10 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C20" s="109" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D20" s="78">
         <v>5.5</v>
@@ -10483,7 +10483,7 @@
         <v>91</v>
       </c>
       <c r="L20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M20" s="97">
         <f t="shared" si="7"/>
@@ -10517,10 +10517,10 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C21" s="109" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D21" s="78">
         <v>1.6</v>
@@ -10547,7 +10547,7 @@
         <v>91</v>
       </c>
       <c r="L21" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M21" s="97">
         <f t="shared" si="7"/>
@@ -10581,10 +10581,10 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C22" s="109" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D22" s="78">
         <v>39.9</v>
@@ -10611,7 +10611,7 @@
         <v>87</v>
       </c>
       <c r="L22" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M22" s="97">
         <f>D22*($J22/100)+D39*($J39/100)</f>
@@ -10645,13 +10645,13 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="87" t="s">
+        <v>213</v>
+      </c>
+      <c r="B23" t="s">
         <v>214</v>
       </c>
-      <c r="B23" t="s">
-        <v>215</v>
-      </c>
       <c r="C23" s="109" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D23" s="78">
         <v>29.7</v>
@@ -10678,7 +10678,7 @@
         <v>88</v>
       </c>
       <c r="L23" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="M23" s="97">
         <f>D23*($J23/100)</f>
@@ -10712,10 +10712,10 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C24" s="109" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D24" s="78">
         <v>1.7</v>
@@ -10742,7 +10742,7 @@
         <v>90</v>
       </c>
       <c r="L24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="M24" s="97">
         <f>D24*($J24/100)</f>
@@ -10776,10 +10776,10 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C25" s="109" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D25" s="78">
         <v>60.4</v>
@@ -10806,7 +10806,7 @@
         <v>11</v>
       </c>
       <c r="L25" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="M25" s="97">
         <f>D25*($J25/100)+D37*($J37/100)</f>
@@ -10840,10 +10840,10 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C26" s="109" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D26" s="78">
         <v>5.2</v>
@@ -10870,7 +10870,7 @@
         <v>76</v>
       </c>
       <c r="L26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M26" s="97">
         <f>D26*($J26/100)</f>
@@ -10904,10 +10904,10 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C27" s="109" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D27" s="78">
         <v>8.6999999999999993</v>
@@ -10934,7 +10934,7 @@
         <v>89</v>
       </c>
       <c r="L27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M27" s="97">
         <f>D27*($J27/100)</f>
@@ -10968,10 +10968,10 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C28" s="109" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D28" s="78">
         <v>188.4</v>
@@ -10998,7 +10998,7 @@
         <v>6.3</v>
       </c>
       <c r="L28" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="M28" s="97">
         <f>D28*($J28/100)+D38*($J38/100)</f>
@@ -11032,10 +11032,10 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C29" s="109" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D29" s="78">
         <v>0</v>
@@ -11062,7 +11062,7 @@
         <v>97</v>
       </c>
       <c r="L29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="M29" s="97">
         <f>D29*($J29/100)</f>
@@ -11096,10 +11096,10 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C30" s="109" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D30" s="78">
         <v>0</v>
@@ -11126,7 +11126,7 @@
         <v>92</v>
       </c>
       <c r="L30" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M30" s="97">
         <f>D30*($J30/100)</f>
@@ -11160,10 +11160,10 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C31" s="109" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D31" s="78">
         <v>2.2000000000000002</v>
@@ -11190,7 +11190,7 @@
         <v>92</v>
       </c>
       <c r="L31" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="M31" s="97">
         <f>D31*($J31/100)</f>
@@ -11224,10 +11224,10 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C32" s="109" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D32" s="78">
         <v>2.2999999999999998</v>
@@ -11254,7 +11254,7 @@
         <v>100</v>
       </c>
       <c r="L32" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M32" s="97">
         <f>D32*($J32/100)</f>
@@ -11288,10 +11288,10 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B33" s="87" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C33" s="141" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D33" s="142">
         <v>62.6</v>
@@ -11316,7 +11316,7 @@
       </c>
       <c r="J33" s="136"/>
       <c r="L33" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="M33" s="101">
         <f>D41*($J41/100)</f>
@@ -11350,10 +11350,10 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B34" s="87" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C34" s="141" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D34" s="142">
         <v>5.8</v>
@@ -11388,10 +11388,10 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B35" s="87" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C35" s="141" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D35" s="142">
         <v>43.3</v>
@@ -11426,10 +11426,10 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C36" s="109" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D36" s="78">
         <v>0</v>
@@ -11467,10 +11467,10 @@
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="87"/>
       <c r="B37" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C37" s="117" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D37" s="118">
         <v>0</v>
@@ -11507,10 +11507,10 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C38" s="109" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D38" s="78">
         <v>0</v>
@@ -11547,10 +11547,10 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C39" s="109" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D39" s="78">
         <v>0</v>
@@ -11587,10 +11587,10 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B40" s="87" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C40" s="145" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D40" s="142">
         <v>0</v>
@@ -11627,10 +11627,10 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C41" s="109" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D41" s="78">
         <v>0</v>
@@ -11667,10 +11667,10 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B42" s="87" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C42" s="146" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D42" s="147">
         <v>0</v>
@@ -11705,7 +11705,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C43" s="121" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D43" s="77">
         <v>2746.2</v>
@@ -11731,7 +11731,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C44" s="107" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D44" s="112">
         <v>4375.1000000000004</v>
@@ -11747,7 +11747,7 @@
       <c r="I44" s="113"/>
       <c r="J44" s="136"/>
       <c r="L44" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M44" s="123">
         <f>SUM(M8:M43)</f>
@@ -11781,7 +11781,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C45" s="114" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D45" s="115">
         <f>SUM(D8:D42)</f>
@@ -11808,7 +11808,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C47" s="137" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L47" s="103"/>
       <c r="M47" s="87"/>
@@ -11817,7 +11817,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C48" s="137" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L48" s="103"/>
       <c r="M48" s="87"/>
@@ -11838,7 +11838,7 @@
     </row>
     <row r="51" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C51" s="138" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D51" s="118"/>
       <c r="E51" s="118"/>
@@ -11850,7 +11850,7 @@
     </row>
     <row r="52" spans="3:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="152" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D52" s="153"/>
       <c r="E52" s="153"/>
@@ -11908,7 +11908,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="K4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -11926,7 +11926,7 @@
         <v>14.6</v>
       </c>
       <c r="K5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -11947,7 +11947,7 @@
         <v>1496.8</v>
       </c>
       <c r="H6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J6">
         <v>18</v>
@@ -11974,7 +11974,7 @@
         <v>374972.8</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J7">
         <f>J4*J5*(1-J6/100)</f>
@@ -12011,7 +12011,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -12034,7 +12034,7 @@
         <v>1.0402648044956555</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E13" s="3">
         <v>2514.0419999999999</v>
@@ -12065,7 +12065,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15" s="3">
         <v>20.3</v>
@@ -12073,7 +12073,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16" s="3">
         <v>5.68</v>
@@ -12098,10 +12098,10 @@
   <sheetData>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -12109,7 +12109,7 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -12117,7 +12117,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -12185,7 +12185,7 @@
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -12238,7 +12238,7 @@
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -12291,7 +12291,7 @@
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" s="2">
         <v>16.88</v>
@@ -12358,7 +12358,7 @@
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C8" s="2">
         <v>11.26</v>
@@ -12425,7 +12425,7 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2">
         <v>57.96</v>
@@ -12492,7 +12492,7 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -12545,7 +12545,7 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -12598,7 +12598,7 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -12651,7 +12651,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -12838,7 +12838,7 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="12">
         <v>1.93</v>
@@ -12905,7 +12905,7 @@
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" s="12">
         <v>0.24</v>
@@ -12972,7 +12972,7 @@
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C18" s="9">
         <v>222</v>
@@ -13039,7 +13039,7 @@
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2">
         <v>0.95</v>
@@ -13106,7 +13106,7 @@
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C20" s="2">
         <v>4.09</v>
@@ -13173,7 +13173,7 @@
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C21" s="2">
         <v>0.76</v>
@@ -13277,19 +13277,19 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="83" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B3" s="83"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="80" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4" s="80">
         <v>0.99999493252819649</v>
@@ -13297,7 +13297,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="80" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B5" s="80">
         <v>0.99998986508207222</v>
@@ -13305,7 +13305,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="80" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B6" s="80">
         <v>0.85713127437951109</v>
@@ -13313,7 +13313,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="80" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B7" s="80">
         <v>0.25677629550654923</v>
@@ -13321,7 +13321,7 @@
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="81" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B8" s="81">
         <v>9</v>
@@ -13329,30 +13329,30 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="82"/>
       <c r="B11" s="82" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="C11" s="82" t="s">
+      <c r="D11" s="82" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="82" t="s">
+      <c r="E11" s="82" t="s">
         <v>130</v>
       </c>
-      <c r="E11" s="82" t="s">
+      <c r="F11" s="82" t="s">
         <v>131</v>
-      </c>
-      <c r="F11" s="82" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="80" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B12" s="80">
         <v>2</v>
@@ -13372,7 +13372,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="80" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B13" s="80">
         <v>7</v>
@@ -13388,7 +13388,7 @@
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B14" s="81">
         <v>9</v>
@@ -13404,33 +13404,33 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="82"/>
       <c r="B16" s="82" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="82" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="82" t="s">
         <v>133</v>
       </c>
-      <c r="C16" s="82" t="s">
-        <v>121</v>
-      </c>
-      <c r="D16" s="82" t="s">
+      <c r="E16" s="82" t="s">
         <v>134</v>
       </c>
-      <c r="E16" s="82" t="s">
+      <c r="F16" s="82" t="s">
         <v>135</v>
       </c>
-      <c r="F16" s="82" t="s">
+      <c r="G16" s="82" t="s">
         <v>136</v>
       </c>
-      <c r="G16" s="82" t="s">
+      <c r="H16" s="82" t="s">
         <v>137</v>
       </c>
-      <c r="H16" s="82" t="s">
+      <c r="I16" s="82" t="s">
         <v>138</v>
-      </c>
-      <c r="I16" s="82" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="80" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B17" s="80">
         <v>0</v>
@@ -13459,7 +13459,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="80" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B18" s="80">
         <v>5.4615384615384617</v>
@@ -13488,7 +13488,7 @@
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="81" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B19" s="81">
         <v>5.7692307692307696E-2</v>
@@ -13517,31 +13517,31 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="82" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="82" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="82" t="s">
+      <c r="C25" s="82" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="82" t="s">
+      <c r="D25" s="82" t="s">
         <v>143</v>
       </c>
-      <c r="D25" s="82" t="s">
-        <v>144</v>
-      </c>
       <c r="F25" s="82" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G25" s="82" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -13745,42 +13745,42 @@
   <sheetData>
     <row r="2" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>104</v>
+      </c>
+      <c r="O2" t="s">
         <v>105</v>
-      </c>
-      <c r="O2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="3" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
       <c r="E3" s="25"/>
       <c r="O3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="2:17" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="D4" s="17" t="s">
         <v>86</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>87</v>
       </c>
       <c r="E4" s="18"/>
       <c r="O4" s="77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P4" s="77" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q4" s="77" t="s">
         <v>108</v>
-      </c>
-      <c r="Q4" s="77" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
@@ -13983,22 +13983,22 @@
         <v>60</v>
       </c>
       <c r="C15" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="30" t="s">
         <v>89</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>90</v>
       </c>
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C16" s="24"/>
       <c r="D16" s="24"/>
       <c r="E16" s="24"/>
       <c r="O16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
@@ -14007,24 +14007,24 @@
       <c r="D17" s="23"/>
       <c r="E17" s="23"/>
       <c r="O17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="2:20" ht="30" x14ac:dyDescent="0.25">
       <c r="O18" s="79" t="s">
+        <v>112</v>
+      </c>
+      <c r="P18" s="79" t="s">
         <v>113</v>
       </c>
-      <c r="P18" s="79" t="s">
+      <c r="Q18" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="R18" s="79" t="s">
+        <v>108</v>
+      </c>
+      <c r="S18" s="79" t="s">
         <v>114</v>
-      </c>
-      <c r="Q18" s="79" t="s">
-        <v>108</v>
-      </c>
-      <c r="R18" s="79" t="s">
-        <v>109</v>
-      </c>
-      <c r="S18" s="79" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.25">
@@ -14067,7 +14067,7 @@
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O21">
         <v>10</v>
@@ -14089,7 +14089,7 @@
     </row>
     <row r="22" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" s="39"/>
       <c r="D22" s="39"/>
@@ -14118,16 +14118,16 @@
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="40"/>
       <c r="C23" s="161" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D23" s="163" t="s">
+        <v>85</v>
+      </c>
+      <c r="E23" s="156" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="156" t="s">
-        <v>87</v>
-      </c>
       <c r="F23" s="158" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G23" s="160"/>
       <c r="H23" s="31"/>
@@ -14205,7 +14205,7 @@
     </row>
     <row r="26" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="155" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C26" s="155"/>
       <c r="D26" s="155"/>
@@ -14303,19 +14303,19 @@
       <c r="G29" s="43"/>
       <c r="H29" s="86"/>
       <c r="O29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="P29" s="84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="Q29" s="84">
         <v>5.46</v>
       </c>
       <c r="R29" s="85" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="S29" s="84" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="T29">
         <v>5.8000000000000003E-2</v>
@@ -14340,7 +14340,7 @@
       <c r="G30" s="43"/>
       <c r="H30" s="86"/>
       <c r="O30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.25">
@@ -14415,7 +14415,7 @@
     </row>
     <row r="35" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="155" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C35" s="155"/>
       <c r="D35" s="155"/>
@@ -14538,14 +14538,14 @@
     </row>
     <row r="42" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B42" s="35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C42" s="36"/>
       <c r="D42" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F42" s="36"/>
       <c r="G42" s="43"/>
@@ -14553,7 +14553,7 @@
     </row>
     <row r="43" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="46" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C43" s="45"/>
       <c r="D43" s="45"/>
@@ -14566,17 +14566,17 @@
     </row>
     <row r="44" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="67" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C47" s="67"/>
       <c r="D47" s="67"/>
@@ -14584,13 +14584,13 @@
     </row>
     <row r="48" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B48" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C48" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="D48" s="16" t="s">
         <v>86</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>87</v>
       </c>
       <c r="E48" s="18"/>
     </row>
@@ -14656,7 +14656,7 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="75" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C54" s="75"/>
       <c r="D54" s="75"/>
@@ -14752,7 +14752,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>